<commit_message>
Se modificó plantilla excel
</commit_message>
<xml_diff>
--- a/plantillas/template.xlsx
+++ b/plantillas/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/02a88c3211e78dcc/Escritorio/Iacc/proyectos/SDW_V2/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="13_ncr:1_{31C7B298-62C6-4CC3-9913-170867C88746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CD01521-6FED-47B7-B38C-4C805A875D58}"/>
+  <xr:revisionPtr revIDLastSave="89" documentId="13_ncr:1_{31C7B298-62C6-4CC3-9913-170867C88746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{445FB2FF-28A7-4F7C-A1C4-9D2E64D72A16}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ORIGINAL" sheetId="9" r:id="rId1"/>
@@ -222,10 +222,10 @@
     <t>(Cubic Meter)</t>
   </si>
   <si>
-    <t xml:space="preserve">              SDW SHIPPING B.V. KORTE BEESTENMARTKT 2-A      </t>
-  </si>
-  <si>
-    <t xml:space="preserve">              2512 GP DEN HAAG THE NETHERLANDS</t>
+    <t xml:space="preserve">SDW SHIPPING B.V. KORTE BEESTENMARTKT 2-A      </t>
+  </si>
+  <si>
+    <t>2512 GP DEN HAAG THE NETHERLANDS</t>
   </si>
 </sst>
 </file>
@@ -807,6 +807,48 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -846,54 +888,42 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -908,36 +938,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1794,24 +1794,24 @@
       <c r="F9" s="17"/>
     </row>
     <row r="10" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="118" t="s">
+      <c r="A10" s="132" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="119"/>
-      <c r="C10" s="120"/>
-      <c r="D10" s="130"/>
-      <c r="E10" s="131"/>
-      <c r="F10" s="132"/>
+      <c r="B10" s="133"/>
+      <c r="C10" s="134"/>
+      <c r="D10" s="117"/>
+      <c r="E10" s="118"/>
+      <c r="F10" s="119"/>
     </row>
     <row r="11" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="118" t="s">
+      <c r="A11" s="132" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="119"/>
-      <c r="C11" s="120"/>
-      <c r="D11" s="130"/>
-      <c r="E11" s="131"/>
-      <c r="F11" s="132"/>
+      <c r="B11" s="133"/>
+      <c r="C11" s="134"/>
+      <c r="D11" s="117"/>
+      <c r="E11" s="118"/>
+      <c r="F11" s="119"/>
     </row>
     <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="28"/>
@@ -1847,17 +1847,17 @@
         <v>5</v>
       </c>
       <c r="C15" s="20"/>
-      <c r="D15" s="133"/>
+      <c r="D15" s="120"/>
       <c r="E15" s="104"/>
-      <c r="F15" s="134"/>
+      <c r="F15" s="121"/>
     </row>
     <row r="16" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="33"/>
       <c r="B16" s="22"/>
       <c r="C16" s="23"/>
-      <c r="D16" s="135"/>
-      <c r="E16" s="136"/>
-      <c r="F16" s="137"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="123"/>
+      <c r="F16" s="124"/>
     </row>
     <row r="17" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
@@ -1872,33 +1872,33 @@
       <c r="F17" s="17"/>
     </row>
     <row r="18" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="155"/>
-      <c r="B18" s="156"/>
-      <c r="C18" s="157"/>
-      <c r="D18" s="138"/>
-      <c r="E18" s="139"/>
-      <c r="F18" s="140"/>
+      <c r="A18" s="150"/>
+      <c r="B18" s="151"/>
+      <c r="C18" s="152"/>
+      <c r="D18" s="125"/>
+      <c r="E18" s="126"/>
+      <c r="F18" s="127"/>
     </row>
     <row r="19" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="155"/>
-      <c r="B19" s="156"/>
-      <c r="C19" s="157"/>
-      <c r="D19" s="138"/>
-      <c r="E19" s="139"/>
-      <c r="F19" s="140"/>
+      <c r="A19" s="150"/>
+      <c r="B19" s="151"/>
+      <c r="C19" s="152"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="126"/>
+      <c r="F19" s="127"/>
     </row>
     <row r="20" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="155"/>
-      <c r="B20" s="156"/>
-      <c r="C20" s="157"/>
-      <c r="D20" s="141"/>
-      <c r="E20" s="142"/>
-      <c r="F20" s="143"/>
+      <c r="A20" s="150"/>
+      <c r="B20" s="151"/>
+      <c r="C20" s="152"/>
+      <c r="D20" s="128"/>
+      <c r="E20" s="129"/>
+      <c r="F20" s="130"/>
     </row>
     <row r="21" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="155"/>
-      <c r="B21" s="156"/>
-      <c r="C21" s="157"/>
+      <c r="A21" s="150"/>
+      <c r="B21" s="151"/>
+      <c r="C21" s="152"/>
       <c r="D21" s="24" t="s">
         <v>51</v>
       </c>
@@ -1906,25 +1906,25 @@
       <c r="F21" s="17"/>
     </row>
     <row r="22" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="124"/>
-      <c r="B22" s="125"/>
-      <c r="C22" s="126"/>
+      <c r="A22" s="138"/>
+      <c r="B22" s="139"/>
+      <c r="C22" s="140"/>
       <c r="D22" s="18"/>
       <c r="E22" s="1"/>
       <c r="F22" s="20"/>
     </row>
     <row r="23" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="124"/>
-      <c r="B23" s="125"/>
-      <c r="C23" s="126"/>
+      <c r="A23" s="138"/>
+      <c r="B23" s="139"/>
+      <c r="C23" s="140"/>
       <c r="D23" s="18"/>
       <c r="E23" s="1"/>
       <c r="F23" s="20"/>
     </row>
     <row r="24" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="147"/>
-      <c r="B24" s="148"/>
-      <c r="C24" s="149"/>
+      <c r="A24" s="157"/>
+      <c r="B24" s="158"/>
+      <c r="C24" s="159"/>
       <c r="D24" s="21"/>
       <c r="E24" s="22"/>
       <c r="F24" s="23"/>
@@ -1942,57 +1942,57 @@
       <c r="F25" s="112"/>
     </row>
     <row r="26" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="121"/>
-      <c r="B26" s="122"/>
-      <c r="C26" s="123"/>
+      <c r="A26" s="135"/>
+      <c r="B26" s="136"/>
+      <c r="C26" s="137"/>
       <c r="D26" s="113"/>
       <c r="E26" s="105"/>
       <c r="F26" s="103"/>
     </row>
     <row r="27" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="124"/>
-      <c r="B27" s="125"/>
-      <c r="C27" s="126"/>
+      <c r="A27" s="138"/>
+      <c r="B27" s="139"/>
+      <c r="C27" s="140"/>
       <c r="D27" s="113"/>
       <c r="E27" s="105"/>
       <c r="F27" s="103"/>
     </row>
     <row r="28" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="124"/>
-      <c r="B28" s="125"/>
-      <c r="C28" s="126"/>
+      <c r="A28" s="138"/>
+      <c r="B28" s="139"/>
+      <c r="C28" s="140"/>
       <c r="D28" s="113"/>
       <c r="E28" s="105"/>
       <c r="F28" s="103"/>
     </row>
     <row r="29" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="124"/>
-      <c r="B29" s="125"/>
-      <c r="C29" s="126"/>
+      <c r="A29" s="138"/>
+      <c r="B29" s="139"/>
+      <c r="C29" s="140"/>
       <c r="D29" s="113"/>
       <c r="E29" s="105"/>
       <c r="F29" s="103"/>
     </row>
     <row r="30" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="124"/>
-      <c r="B30" s="125"/>
-      <c r="C30" s="126"/>
+      <c r="A30" s="138"/>
+      <c r="B30" s="139"/>
+      <c r="C30" s="140"/>
       <c r="D30" s="113"/>
       <c r="E30" s="105"/>
       <c r="F30" s="103"/>
     </row>
     <row r="31" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="124"/>
-      <c r="B31" s="125"/>
-      <c r="C31" s="126"/>
+      <c r="A31" s="138"/>
+      <c r="B31" s="139"/>
+      <c r="C31" s="140"/>
       <c r="D31" s="113"/>
       <c r="E31" s="105"/>
       <c r="F31" s="103"/>
     </row>
     <row r="32" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="127"/>
-      <c r="B32" s="128"/>
-      <c r="C32" s="129"/>
+      <c r="A32" s="141"/>
+      <c r="B32" s="142"/>
+      <c r="C32" s="143"/>
       <c r="D32" s="113"/>
       <c r="E32" s="105"/>
       <c r="F32" s="103"/>
@@ -2018,7 +2018,7 @@
       <c r="F34" s="116"/>
     </row>
     <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="117" t="s">
+      <c r="A35" s="131" t="s">
         <v>47</v>
       </c>
       <c r="B35" s="112"/>
@@ -2032,12 +2032,12 @@
       <c r="F35" s="17"/>
     </row>
     <row r="36" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="150"/>
+      <c r="A36" s="160"/>
       <c r="B36" s="116"/>
       <c r="C36" s="47"/>
-      <c r="D36" s="135"/>
-      <c r="E36" s="136"/>
-      <c r="F36" s="137"/>
+      <c r="D36" s="122"/>
+      <c r="E36" s="123"/>
+      <c r="F36" s="124"/>
     </row>
     <row r="37" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="24" t="s">
@@ -2058,13 +2058,13 @@
       <c r="B38" s="145"/>
       <c r="C38" s="49"/>
       <c r="D38" s="144"/>
-      <c r="E38" s="146"/>
+      <c r="E38" s="156"/>
       <c r="F38" s="145"/>
     </row>
     <row r="39" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
-      <c r="C39" s="158"/>
+      <c r="C39" s="153"/>
       <c r="D39" s="105"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
@@ -2076,7 +2076,7 @@
       <c r="B40" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="159" t="s">
+      <c r="C40" s="154" t="s">
         <v>9</v>
       </c>
       <c r="D40" s="112"/>
@@ -2092,7 +2092,7 @@
         <v>7</v>
       </c>
       <c r="B41" s="51"/>
-      <c r="C41" s="160"/>
+      <c r="C41" s="155"/>
       <c r="D41" s="116"/>
       <c r="E41" s="51" t="s">
         <v>59</v>
@@ -2308,8 +2308,8 @@
       <c r="F66" s="48"/>
     </row>
     <row r="67" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="151"/>
-      <c r="B67" s="152"/>
+      <c r="A67" s="146"/>
+      <c r="B67" s="147"/>
       <c r="C67" s="90"/>
       <c r="D67" s="91"/>
       <c r="E67" s="11"/>
@@ -2346,8 +2346,8 @@
       <c r="F70" s="74"/>
     </row>
     <row r="71" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="153"/>
-      <c r="B71" s="154"/>
+      <c r="A71" s="148"/>
+      <c r="B71" s="149"/>
       <c r="C71" s="97"/>
       <c r="D71" s="10"/>
       <c r="E71" s="10"/>
@@ -2396,11 +2396,6 @@
     <mergeCell ref="A67:B67"/>
     <mergeCell ref="A71:B71"/>
     <mergeCell ref="D72:F72"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="D36:F36"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="D38:F38"/>
     <mergeCell ref="C39:D39"/>
     <mergeCell ref="D25:F34"/>
     <mergeCell ref="A26:C26"/>
@@ -2411,11 +2406,11 @@
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="A32:C32"/>
     <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="D38:F38"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="D15:F15"/>
     <mergeCell ref="D16:F16"/>
@@ -2423,13 +2418,18 @@
     <mergeCell ref="D18:F18"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="D19:F19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
     <mergeCell ref="D2:E5"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="D10:F10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0" bottom="0" header="0" footer="0"/>
@@ -2541,24 +2541,24 @@
       <c r="F9" s="17"/>
     </row>
     <row r="10" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="118" t="s">
+      <c r="A10" s="132" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="119"/>
-      <c r="C10" s="120"/>
-      <c r="D10" s="130"/>
-      <c r="E10" s="131"/>
-      <c r="F10" s="132"/>
+      <c r="B10" s="133"/>
+      <c r="C10" s="134"/>
+      <c r="D10" s="117"/>
+      <c r="E10" s="118"/>
+      <c r="F10" s="119"/>
     </row>
     <row r="11" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="118" t="s">
+      <c r="A11" s="132" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="119"/>
-      <c r="C11" s="120"/>
-      <c r="D11" s="130"/>
-      <c r="E11" s="131"/>
-      <c r="F11" s="132"/>
+      <c r="B11" s="133"/>
+      <c r="C11" s="134"/>
+      <c r="D11" s="117"/>
+      <c r="E11" s="118"/>
+      <c r="F11" s="119"/>
     </row>
     <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="28"/>
@@ -2594,17 +2594,17 @@
         <v>5</v>
       </c>
       <c r="C15" s="20"/>
-      <c r="D15" s="133"/>
+      <c r="D15" s="120"/>
       <c r="E15" s="104"/>
-      <c r="F15" s="134"/>
+      <c r="F15" s="121"/>
     </row>
     <row r="16" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="33"/>
       <c r="B16" s="22"/>
       <c r="C16" s="23"/>
-      <c r="D16" s="135"/>
-      <c r="E16" s="136"/>
-      <c r="F16" s="137"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="123"/>
+      <c r="F16" s="124"/>
     </row>
     <row r="17" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
@@ -2619,33 +2619,33 @@
       <c r="F17" s="17"/>
     </row>
     <row r="18" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="155"/>
-      <c r="B18" s="156"/>
-      <c r="C18" s="157"/>
-      <c r="D18" s="138"/>
-      <c r="E18" s="139"/>
-      <c r="F18" s="140"/>
+      <c r="A18" s="150"/>
+      <c r="B18" s="151"/>
+      <c r="C18" s="152"/>
+      <c r="D18" s="125"/>
+      <c r="E18" s="126"/>
+      <c r="F18" s="127"/>
     </row>
     <row r="19" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="155"/>
-      <c r="B19" s="156"/>
-      <c r="C19" s="157"/>
-      <c r="D19" s="138"/>
-      <c r="E19" s="139"/>
-      <c r="F19" s="140"/>
+      <c r="A19" s="150"/>
+      <c r="B19" s="151"/>
+      <c r="C19" s="152"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="126"/>
+      <c r="F19" s="127"/>
     </row>
     <row r="20" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="155"/>
-      <c r="B20" s="156"/>
-      <c r="C20" s="157"/>
-      <c r="D20" s="141"/>
-      <c r="E20" s="142"/>
-      <c r="F20" s="143"/>
+      <c r="A20" s="150"/>
+      <c r="B20" s="151"/>
+      <c r="C20" s="152"/>
+      <c r="D20" s="128"/>
+      <c r="E20" s="129"/>
+      <c r="F20" s="130"/>
     </row>
     <row r="21" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="155"/>
-      <c r="B21" s="156"/>
-      <c r="C21" s="157"/>
+      <c r="A21" s="150"/>
+      <c r="B21" s="151"/>
+      <c r="C21" s="152"/>
       <c r="D21" s="24" t="s">
         <v>51</v>
       </c>
@@ -2653,25 +2653,25 @@
       <c r="F21" s="17"/>
     </row>
     <row r="22" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="124"/>
-      <c r="B22" s="125"/>
-      <c r="C22" s="126"/>
+      <c r="A22" s="138"/>
+      <c r="B22" s="139"/>
+      <c r="C22" s="140"/>
       <c r="D22" s="18"/>
       <c r="E22" s="1"/>
       <c r="F22" s="20"/>
     </row>
     <row r="23" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="124"/>
-      <c r="B23" s="125"/>
-      <c r="C23" s="126"/>
+      <c r="A23" s="138"/>
+      <c r="B23" s="139"/>
+      <c r="C23" s="140"/>
       <c r="D23" s="18"/>
       <c r="E23" s="1"/>
       <c r="F23" s="20"/>
     </row>
     <row r="24" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="147"/>
-      <c r="B24" s="148"/>
-      <c r="C24" s="149"/>
+      <c r="A24" s="157"/>
+      <c r="B24" s="158"/>
+      <c r="C24" s="159"/>
       <c r="D24" s="21"/>
       <c r="E24" s="22"/>
       <c r="F24" s="23"/>
@@ -2689,57 +2689,57 @@
       <c r="F25" s="112"/>
     </row>
     <row r="26" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="121"/>
-      <c r="B26" s="122"/>
-      <c r="C26" s="123"/>
+      <c r="A26" s="135"/>
+      <c r="B26" s="136"/>
+      <c r="C26" s="137"/>
       <c r="D26" s="113"/>
       <c r="E26" s="105"/>
       <c r="F26" s="103"/>
     </row>
     <row r="27" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="124"/>
-      <c r="B27" s="125"/>
-      <c r="C27" s="126"/>
+      <c r="A27" s="138"/>
+      <c r="B27" s="139"/>
+      <c r="C27" s="140"/>
       <c r="D27" s="113"/>
       <c r="E27" s="105"/>
       <c r="F27" s="103"/>
     </row>
     <row r="28" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="124"/>
-      <c r="B28" s="125"/>
-      <c r="C28" s="126"/>
+      <c r="A28" s="138"/>
+      <c r="B28" s="139"/>
+      <c r="C28" s="140"/>
       <c r="D28" s="113"/>
       <c r="E28" s="105"/>
       <c r="F28" s="103"/>
     </row>
     <row r="29" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="124"/>
-      <c r="B29" s="125"/>
-      <c r="C29" s="126"/>
+      <c r="A29" s="138"/>
+      <c r="B29" s="139"/>
+      <c r="C29" s="140"/>
       <c r="D29" s="113"/>
       <c r="E29" s="105"/>
       <c r="F29" s="103"/>
     </row>
     <row r="30" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="124"/>
-      <c r="B30" s="125"/>
-      <c r="C30" s="126"/>
+      <c r="A30" s="138"/>
+      <c r="B30" s="139"/>
+      <c r="C30" s="140"/>
       <c r="D30" s="113"/>
       <c r="E30" s="105"/>
       <c r="F30" s="103"/>
     </row>
     <row r="31" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="124"/>
-      <c r="B31" s="125"/>
-      <c r="C31" s="126"/>
+      <c r="A31" s="138"/>
+      <c r="B31" s="139"/>
+      <c r="C31" s="140"/>
       <c r="D31" s="113"/>
       <c r="E31" s="105"/>
       <c r="F31" s="103"/>
     </row>
     <row r="32" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="127"/>
-      <c r="B32" s="128"/>
-      <c r="C32" s="129"/>
+      <c r="A32" s="141"/>
+      <c r="B32" s="142"/>
+      <c r="C32" s="143"/>
       <c r="D32" s="113"/>
       <c r="E32" s="105"/>
       <c r="F32" s="103"/>
@@ -2765,7 +2765,7 @@
       <c r="F34" s="116"/>
     </row>
     <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="117" t="s">
+      <c r="A35" s="131" t="s">
         <v>47</v>
       </c>
       <c r="B35" s="112"/>
@@ -2779,12 +2779,12 @@
       <c r="F35" s="17"/>
     </row>
     <row r="36" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="150"/>
+      <c r="A36" s="160"/>
       <c r="B36" s="116"/>
       <c r="C36" s="47"/>
-      <c r="D36" s="135"/>
-      <c r="E36" s="136"/>
-      <c r="F36" s="137"/>
+      <c r="D36" s="122"/>
+      <c r="E36" s="123"/>
+      <c r="F36" s="124"/>
     </row>
     <row r="37" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="24" t="s">
@@ -2805,13 +2805,13 @@
       <c r="B38" s="145"/>
       <c r="C38" s="49"/>
       <c r="D38" s="144"/>
-      <c r="E38" s="146"/>
+      <c r="E38" s="156"/>
       <c r="F38" s="145"/>
     </row>
     <row r="39" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
-      <c r="C39" s="158"/>
+      <c r="C39" s="153"/>
       <c r="D39" s="105"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
@@ -2823,7 +2823,7 @@
       <c r="B40" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="159" t="s">
+      <c r="C40" s="154" t="s">
         <v>9</v>
       </c>
       <c r="D40" s="112"/>
@@ -2839,7 +2839,7 @@
         <v>7</v>
       </c>
       <c r="B41" s="51"/>
-      <c r="C41" s="160"/>
+      <c r="C41" s="155"/>
       <c r="D41" s="116"/>
       <c r="E41" s="51" t="s">
         <v>59</v>
@@ -3055,8 +3055,8 @@
       <c r="F66" s="48"/>
     </row>
     <row r="67" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="151"/>
-      <c r="B67" s="152"/>
+      <c r="A67" s="146"/>
+      <c r="B67" s="147"/>
       <c r="C67" s="90"/>
       <c r="D67" s="91"/>
       <c r="E67" s="11"/>
@@ -3093,8 +3093,8 @@
       <c r="F70" s="74"/>
     </row>
     <row r="71" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="153"/>
-      <c r="B71" s="154"/>
+      <c r="A71" s="148"/>
+      <c r="B71" s="149"/>
       <c r="C71" s="97"/>
       <c r="D71" s="10"/>
       <c r="E71" s="10"/>
@@ -3505,7 +3505,7 @@
       <c r="F34" s="116"/>
     </row>
     <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="117" t="s">
+      <c r="A35" s="131" t="s">
         <v>47</v>
       </c>
       <c r="B35" s="112"/>
@@ -3519,7 +3519,7 @@
       <c r="F35" s="17"/>
     </row>
     <row r="36" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="150"/>
+      <c r="A36" s="160"/>
       <c r="B36" s="116"/>
       <c r="C36" s="47"/>
       <c r="D36" s="21"/>
@@ -3551,7 +3551,7 @@
     <row r="39" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
-      <c r="C39" s="158"/>
+      <c r="C39" s="153"/>
       <c r="D39" s="105"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
@@ -3563,7 +3563,7 @@
       <c r="B40" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="159" t="s">
+      <c r="C40" s="154" t="s">
         <v>9</v>
       </c>
       <c r="D40" s="112"/>
@@ -3579,7 +3579,7 @@
         <v>7</v>
       </c>
       <c r="B41" s="51"/>
-      <c r="C41" s="160"/>
+      <c r="C41" s="155"/>
       <c r="D41" s="116"/>
       <c r="E41" s="51" t="s">
         <v>59</v>
@@ -4252,7 +4252,7 @@
     </row>
     <row r="40" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="117" t="s">
+      <c r="B40" s="131" t="s">
         <v>35</v>
       </c>
       <c r="C40" s="112"/>
@@ -4267,7 +4267,7 @@
     </row>
     <row r="41" spans="1:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
-      <c r="B41" s="150"/>
+      <c r="B41" s="160"/>
       <c r="C41" s="116"/>
       <c r="D41" s="47"/>
       <c r="E41" s="21"/>
@@ -4302,7 +4302,7 @@
       <c r="A44" s="1"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
-      <c r="D44" s="158"/>
+      <c r="D44" s="153"/>
       <c r="E44" s="105"/>
       <c r="F44" s="7"/>
       <c r="G44" s="7"/>
@@ -4315,7 +4315,7 @@
       <c r="C45" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="D45" s="159" t="s">
+      <c r="D45" s="154" t="s">
         <v>9</v>
       </c>
       <c r="E45" s="112"/>
@@ -4334,7 +4334,7 @@
       <c r="C46" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="D46" s="160" t="s">
+      <c r="D46" s="155" t="s">
         <v>14</v>
       </c>
       <c r="E46" s="116"/>

</xml_diff>

<commit_message>
Modificaciones según excel final de cliente
</commit_message>
<xml_diff>
--- a/plantillas/template.xlsx
+++ b/plantillas/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/02a88c3211e78dcc/Escritorio/Iacc/proyectos/SDW_V2/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="89" documentId="13_ncr:1_{31C7B298-62C6-4CC3-9913-170867C88746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{445FB2FF-28A7-4F7C-A1C4-9D2E64D72A16}"/>
+  <xr:revisionPtr revIDLastSave="255" documentId="13_ncr:1_{31C7B298-62C6-4CC3-9913-170867C88746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC787503-3612-4A83-8CBD-4FBAB924B17F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ORIGINAL" sheetId="9" r:id="rId1"/>
@@ -236,7 +236,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="_(&quot;B&quot;* #,##0.00_);_(&quot;B&quot;* \(#,##0.00\);_(&quot;B&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="31" x14ac:knownFonts="1">
+  <fonts count="40" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -440,6 +440,60 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -595,7 +649,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="232">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -778,35 +832,289 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="38" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="34" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="34" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="38" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="38" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="38" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="34" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -822,15 +1130,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -847,96 +1146,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1001,7 +1210,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7667625" y="16554450"/>
+          <a:off x="7667625" y="17297400"/>
           <a:ext cx="4667250" cy="38100"/>
           <a:chOff x="3012375" y="3780000"/>
           <a:chExt cx="4667250" cy="0"/>
@@ -1091,7 +1300,7 @@
       <xdr:col>4</xdr:col>
       <xdr:colOff>1981199</xdr:colOff>
       <xdr:row>72</xdr:row>
-      <xdr:rowOff>196227</xdr:rowOff>
+      <xdr:rowOff>139077</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1715,10 +1924,10 @@
       <c r="A2" s="15"/>
       <c r="B2" s="16"/>
       <c r="C2" s="17"/>
-      <c r="D2" s="107" t="s">
+      <c r="D2" s="188" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="108"/>
+      <c r="E2" s="163"/>
       <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
@@ -1727,8 +1936,8 @@
       <c r="C3" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="105"/>
-      <c r="E3" s="105"/>
+      <c r="D3" s="148"/>
+      <c r="E3" s="148"/>
       <c r="F3" s="20"/>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1737,8 +1946,8 @@
       <c r="C4" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="105"/>
-      <c r="E4" s="105"/>
+      <c r="D4" s="148"/>
+      <c r="E4" s="148"/>
       <c r="F4" s="20"/>
     </row>
     <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1747,8 +1956,8 @@
       <c r="C5" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="105"/>
-      <c r="E5" s="105"/>
+      <c r="D5" s="148"/>
+      <c r="E5" s="148"/>
       <c r="F5" s="20"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1757,20 +1966,20 @@
       <c r="C6" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="109" t="s">
+      <c r="D6" s="189" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="105"/>
+      <c r="E6" s="148"/>
       <c r="F6" s="20"/>
     </row>
     <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="18"/>
       <c r="B7" s="1"/>
       <c r="C7" s="20"/>
-      <c r="D7" s="110" t="s">
+      <c r="D7" s="190" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="105"/>
+      <c r="E7" s="148"/>
       <c r="F7" s="20"/>
     </row>
     <row r="8" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -1781,7 +1990,7 @@
       <c r="E8" s="22"/>
       <c r="F8" s="23"/>
     </row>
-    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A9" s="24" t="s">
         <v>54</v>
       </c>
@@ -1790,238 +1999,238 @@
       <c r="D9" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="16"/>
-      <c r="F9" s="17"/>
-    </row>
-    <row r="10" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="132" t="s">
+      <c r="E9" s="113"/>
+      <c r="F9" s="114"/>
+    </row>
+    <row r="10" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="167" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="133"/>
-      <c r="C10" s="134"/>
-      <c r="D10" s="117"/>
-      <c r="E10" s="118"/>
-      <c r="F10" s="119"/>
-    </row>
-    <row r="11" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="132" t="s">
+      <c r="B10" s="168"/>
+      <c r="C10" s="169"/>
+      <c r="D10" s="167"/>
+      <c r="E10" s="168"/>
+      <c r="F10" s="169"/>
+    </row>
+    <row r="11" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="167" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="133"/>
-      <c r="C11" s="134"/>
-      <c r="D11" s="117"/>
-      <c r="E11" s="118"/>
-      <c r="F11" s="119"/>
-    </row>
-    <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="20"/>
+      <c r="B11" s="168"/>
+      <c r="C11" s="169"/>
+      <c r="D11" s="167"/>
+      <c r="E11" s="168"/>
+      <c r="F11" s="169"/>
+    </row>
+    <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="104"/>
+      <c r="B12" s="105"/>
+      <c r="C12" s="106"/>
       <c r="D12" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="20"/>
-    </row>
-    <row r="13" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="31"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="23"/>
-    </row>
-    <row r="14" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="28"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="20"/>
+      <c r="E12" s="105"/>
+      <c r="F12" s="106"/>
+    </row>
+    <row r="13" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="107"/>
+      <c r="B13" s="105"/>
+      <c r="C13" s="106"/>
+      <c r="D13" s="115"/>
+      <c r="E13" s="111"/>
+      <c r="F13" s="112"/>
+    </row>
+    <row r="14" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="104"/>
+      <c r="B14" s="105"/>
+      <c r="C14" s="106"/>
       <c r="D14" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="16"/>
-      <c r="F14" s="17"/>
-    </row>
-    <row r="15" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="32"/>
-      <c r="B15" s="4" t="s">
+      <c r="E14" s="113"/>
+      <c r="F14" s="114"/>
+    </row>
+    <row r="15" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="108"/>
+      <c r="B15" s="109" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="120"/>
-      <c r="E15" s="104"/>
-      <c r="F15" s="121"/>
-    </row>
-    <row r="16" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="33"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
-      <c r="F16" s="124"/>
-    </row>
-    <row r="17" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C15" s="106"/>
+      <c r="D15" s="182"/>
+      <c r="E15" s="183"/>
+      <c r="F15" s="184"/>
+    </row>
+    <row r="16" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="110"/>
+      <c r="B16" s="111"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="173"/>
+      <c r="E16" s="178"/>
+      <c r="F16" s="174"/>
+    </row>
+    <row r="17" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A17" s="24" t="s">
         <v>56</v>
       </c>
       <c r="B17" s="25"/>
-      <c r="C17" s="26"/>
+      <c r="C17" s="118"/>
       <c r="D17" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="E17" s="16"/>
-      <c r="F17" s="17"/>
-    </row>
-    <row r="18" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="150"/>
-      <c r="B18" s="151"/>
-      <c r="C18" s="152"/>
-      <c r="D18" s="125"/>
-      <c r="E18" s="126"/>
-      <c r="F18" s="127"/>
-    </row>
-    <row r="19" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="150"/>
-      <c r="B19" s="151"/>
-      <c r="C19" s="152"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="126"/>
-      <c r="F19" s="127"/>
-    </row>
-    <row r="20" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="150"/>
-      <c r="B20" s="151"/>
-      <c r="C20" s="152"/>
-      <c r="D20" s="128"/>
-      <c r="E20" s="129"/>
-      <c r="F20" s="130"/>
-    </row>
-    <row r="21" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="150"/>
-      <c r="B21" s="151"/>
-      <c r="C21" s="152"/>
+      <c r="E17" s="113"/>
+      <c r="F17" s="114"/>
+    </row>
+    <row r="18" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="185"/>
+      <c r="B18" s="186"/>
+      <c r="C18" s="187"/>
+      <c r="D18" s="182"/>
+      <c r="E18" s="183"/>
+      <c r="F18" s="184"/>
+    </row>
+    <row r="19" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="185"/>
+      <c r="B19" s="186"/>
+      <c r="C19" s="187"/>
+      <c r="D19" s="182"/>
+      <c r="E19" s="183"/>
+      <c r="F19" s="184"/>
+    </row>
+    <row r="20" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="185"/>
+      <c r="B20" s="186"/>
+      <c r="C20" s="187"/>
+      <c r="D20" s="173"/>
+      <c r="E20" s="178"/>
+      <c r="F20" s="174"/>
+    </row>
+    <row r="21" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="185"/>
+      <c r="B21" s="186"/>
+      <c r="C21" s="187"/>
       <c r="D21" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="16"/>
-      <c r="F21" s="17"/>
-    </row>
-    <row r="22" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="138"/>
-      <c r="B22" s="139"/>
-      <c r="C22" s="140"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="20"/>
-    </row>
-    <row r="23" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="138"/>
-      <c r="B23" s="139"/>
-      <c r="C23" s="140"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="20"/>
-    </row>
-    <row r="24" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="157"/>
-      <c r="B24" s="158"/>
-      <c r="C24" s="159"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="23"/>
-    </row>
-    <row r="25" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E21" s="113"/>
+      <c r="F21" s="114"/>
+    </row>
+    <row r="22" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="167"/>
+      <c r="B22" s="168"/>
+      <c r="C22" s="169"/>
+      <c r="D22" s="117"/>
+      <c r="E22" s="105"/>
+      <c r="F22" s="106"/>
+    </row>
+    <row r="23" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="167"/>
+      <c r="B23" s="168"/>
+      <c r="C23" s="169"/>
+      <c r="D23" s="117"/>
+      <c r="E23" s="105"/>
+      <c r="F23" s="106"/>
+    </row>
+    <row r="24" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="179"/>
+      <c r="B24" s="180"/>
+      <c r="C24" s="181"/>
+      <c r="D24" s="115"/>
+      <c r="E24" s="111"/>
+      <c r="F24" s="112"/>
+    </row>
+    <row r="25" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A25" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="41"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="111" t="s">
+      <c r="B25" s="113"/>
+      <c r="C25" s="118"/>
+      <c r="D25" s="162" t="s">
         <v>6</v>
       </c>
-      <c r="E25" s="108"/>
-      <c r="F25" s="112"/>
-    </row>
-    <row r="26" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="135"/>
-      <c r="B26" s="136"/>
-      <c r="C26" s="137"/>
-      <c r="D26" s="113"/>
-      <c r="E26" s="105"/>
-      <c r="F26" s="103"/>
-    </row>
-    <row r="27" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="138"/>
-      <c r="B27" s="139"/>
-      <c r="C27" s="140"/>
-      <c r="D27" s="113"/>
-      <c r="E27" s="105"/>
-      <c r="F27" s="103"/>
-    </row>
-    <row r="28" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="138"/>
-      <c r="B28" s="139"/>
-      <c r="C28" s="140"/>
-      <c r="D28" s="113"/>
-      <c r="E28" s="105"/>
-      <c r="F28" s="103"/>
-    </row>
-    <row r="29" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="138"/>
-      <c r="B29" s="139"/>
-      <c r="C29" s="140"/>
-      <c r="D29" s="113"/>
-      <c r="E29" s="105"/>
-      <c r="F29" s="103"/>
-    </row>
-    <row r="30" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="138"/>
-      <c r="B30" s="139"/>
-      <c r="C30" s="140"/>
-      <c r="D30" s="113"/>
-      <c r="E30" s="105"/>
-      <c r="F30" s="103"/>
-    </row>
-    <row r="31" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="138"/>
-      <c r="B31" s="139"/>
-      <c r="C31" s="140"/>
-      <c r="D31" s="113"/>
-      <c r="E31" s="105"/>
-      <c r="F31" s="103"/>
-    </row>
-    <row r="32" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="141"/>
-      <c r="B32" s="142"/>
-      <c r="C32" s="143"/>
-      <c r="D32" s="113"/>
-      <c r="E32" s="105"/>
-      <c r="F32" s="103"/>
-    </row>
-    <row r="33" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E25" s="163"/>
+      <c r="F25" s="151"/>
+    </row>
+    <row r="26" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="167"/>
+      <c r="B26" s="168"/>
+      <c r="C26" s="169"/>
+      <c r="D26" s="164"/>
+      <c r="E26" s="148"/>
+      <c r="F26" s="149"/>
+    </row>
+    <row r="27" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="167"/>
+      <c r="B27" s="168"/>
+      <c r="C27" s="169"/>
+      <c r="D27" s="164"/>
+      <c r="E27" s="148"/>
+      <c r="F27" s="149"/>
+    </row>
+    <row r="28" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="167"/>
+      <c r="B28" s="168"/>
+      <c r="C28" s="169"/>
+      <c r="D28" s="164"/>
+      <c r="E28" s="148"/>
+      <c r="F28" s="149"/>
+    </row>
+    <row r="29" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="167"/>
+      <c r="B29" s="168"/>
+      <c r="C29" s="169"/>
+      <c r="D29" s="164"/>
+      <c r="E29" s="148"/>
+      <c r="F29" s="149"/>
+    </row>
+    <row r="30" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="167"/>
+      <c r="B30" s="168"/>
+      <c r="C30" s="169"/>
+      <c r="D30" s="164"/>
+      <c r="E30" s="148"/>
+      <c r="F30" s="149"/>
+    </row>
+    <row r="31" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="167"/>
+      <c r="B31" s="168"/>
+      <c r="C31" s="169"/>
+      <c r="D31" s="164"/>
+      <c r="E31" s="148"/>
+      <c r="F31" s="149"/>
+    </row>
+    <row r="32" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="170"/>
+      <c r="B32" s="171"/>
+      <c r="C32" s="172"/>
+      <c r="D32" s="164"/>
+      <c r="E32" s="148"/>
+      <c r="F32" s="149"/>
+    </row>
+    <row r="33" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A33" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="16"/>
+      <c r="B33" s="113"/>
       <c r="C33" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="D33" s="113"/>
-      <c r="E33" s="105"/>
-      <c r="F33" s="103"/>
-    </row>
-    <row r="34" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="144"/>
-      <c r="B34" s="145"/>
-      <c r="C34" s="47"/>
-      <c r="D34" s="114"/>
-      <c r="E34" s="115"/>
-      <c r="F34" s="116"/>
-    </row>
-    <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="131" t="s">
+      <c r="D33" s="164"/>
+      <c r="E33" s="148"/>
+      <c r="F33" s="149"/>
+    </row>
+    <row r="34" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="173"/>
+      <c r="B34" s="174"/>
+      <c r="C34" s="123"/>
+      <c r="D34" s="165"/>
+      <c r="E34" s="166"/>
+      <c r="F34" s="153"/>
+    </row>
+    <row r="35" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A35" s="175" t="s">
         <v>47</v>
       </c>
-      <c r="B35" s="112"/>
+      <c r="B35" s="151"/>
       <c r="C35" s="46" t="s">
         <v>48</v>
       </c>
@@ -2029,21 +2238,21 @@
         <v>49</v>
       </c>
       <c r="E35" s="16"/>
-      <c r="F35" s="17"/>
-    </row>
-    <row r="36" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="160"/>
-      <c r="B36" s="116"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="122"/>
-      <c r="E36" s="123"/>
-      <c r="F36" s="124"/>
-    </row>
-    <row r="37" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F35" s="114"/>
+    </row>
+    <row r="36" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="176"/>
+      <c r="B36" s="177"/>
+      <c r="C36" s="103"/>
+      <c r="D36" s="173"/>
+      <c r="E36" s="178"/>
+      <c r="F36" s="174"/>
+    </row>
+    <row r="37" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A37" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="B37" s="48"/>
+      <c r="B37" s="102"/>
       <c r="C37" s="46" t="s">
         <v>45</v>
       </c>
@@ -2051,21 +2260,21 @@
         <v>44</v>
       </c>
       <c r="E37" s="16"/>
-      <c r="F37" s="17"/>
-    </row>
-    <row r="38" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="144"/>
-      <c r="B38" s="145"/>
-      <c r="C38" s="49"/>
-      <c r="D38" s="144"/>
-      <c r="E38" s="156"/>
-      <c r="F38" s="145"/>
+      <c r="F37" s="114"/>
+    </row>
+    <row r="38" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="173"/>
+      <c r="B38" s="174"/>
+      <c r="C38" s="138"/>
+      <c r="D38" s="173"/>
+      <c r="E38" s="178"/>
+      <c r="F38" s="174"/>
     </row>
     <row r="39" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
-      <c r="C39" s="153"/>
-      <c r="D39" s="105"/>
+      <c r="C39" s="161"/>
+      <c r="D39" s="148"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
     </row>
@@ -2076,10 +2285,10 @@
       <c r="B40" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="154" t="s">
+      <c r="C40" s="150" t="s">
         <v>9</v>
       </c>
-      <c r="D40" s="112"/>
+      <c r="D40" s="151"/>
       <c r="E40" s="50" t="s">
         <v>10</v>
       </c>
@@ -2092,8 +2301,8 @@
         <v>7</v>
       </c>
       <c r="B41" s="51"/>
-      <c r="C41" s="155"/>
-      <c r="D41" s="116"/>
+      <c r="C41" s="152"/>
+      <c r="D41" s="153"/>
       <c r="E41" s="51" t="s">
         <v>59</v>
       </c>
@@ -2101,189 +2310,189 @@
         <v>60</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="52"/>
-      <c r="B42" s="53"/>
-      <c r="C42" s="54"/>
-      <c r="D42" s="17"/>
-      <c r="E42" s="53"/>
-      <c r="F42" s="53"/>
-    </row>
-    <row r="43" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="55"/>
-      <c r="B43" s="56"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="57"/>
-      <c r="E43" s="102"/>
-      <c r="F43" s="58"/>
-    </row>
-    <row r="44" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="59"/>
-      <c r="B44" s="60"/>
-      <c r="C44" s="1"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="103"/>
-      <c r="F44" s="60"/>
-    </row>
-    <row r="45" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="55"/>
-      <c r="B45" s="61"/>
-      <c r="C45" s="1"/>
-      <c r="D45" s="20"/>
-      <c r="E45" s="62"/>
-      <c r="F45" s="63"/>
-    </row>
-    <row r="46" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="64"/>
-      <c r="B46" s="60"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="20"/>
-      <c r="E46" s="20"/>
-      <c r="F46" s="20"/>
-    </row>
-    <row r="47" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="55"/>
-      <c r="B47" s="20"/>
-      <c r="C47" s="1"/>
-      <c r="D47" s="20"/>
-      <c r="E47" s="20"/>
-      <c r="F47" s="20"/>
-    </row>
-    <row r="48" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="55"/>
-      <c r="B48" s="20"/>
-      <c r="C48" s="1"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="20"/>
-      <c r="F48" s="20"/>
-    </row>
-    <row r="49" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="55"/>
-      <c r="B49" s="20"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="20"/>
-      <c r="E49" s="20"/>
-      <c r="F49" s="20"/>
-    </row>
-    <row r="50" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="65"/>
-      <c r="B50" s="56"/>
-      <c r="C50" s="1"/>
-      <c r="D50" s="20"/>
-      <c r="E50" s="66"/>
-      <c r="F50" s="60"/>
-    </row>
-    <row r="51" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="65"/>
-      <c r="B51" s="60"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="20"/>
-      <c r="E51" s="66"/>
-      <c r="F51" s="60"/>
-    </row>
-    <row r="52" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="65"/>
-      <c r="B52" s="60"/>
-      <c r="C52" s="1"/>
-      <c r="D52" s="20"/>
-      <c r="E52" s="66"/>
-      <c r="F52" s="60"/>
-    </row>
-    <row r="53" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="65"/>
-      <c r="B53" s="60"/>
-      <c r="C53" s="1"/>
-      <c r="D53" s="20"/>
-      <c r="E53" s="66"/>
-      <c r="F53" s="60"/>
-    </row>
-    <row r="54" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="65"/>
-      <c r="B54" s="60"/>
-      <c r="C54" s="1"/>
-      <c r="D54" s="20"/>
-      <c r="E54" s="66"/>
-      <c r="F54" s="60"/>
-    </row>
-    <row r="55" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="65"/>
-      <c r="B55" s="56"/>
-      <c r="C55" s="1"/>
-      <c r="D55" s="20"/>
-      <c r="E55" s="66"/>
-      <c r="F55" s="60"/>
-    </row>
-    <row r="56" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="65"/>
-      <c r="B56" s="56"/>
-      <c r="C56" s="1"/>
-      <c r="D56" s="20"/>
-      <c r="E56" s="20"/>
-      <c r="F56" s="66"/>
-    </row>
-    <row r="57" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="65"/>
-      <c r="B57" s="20"/>
-      <c r="C57" s="1"/>
-      <c r="D57" s="20"/>
-      <c r="E57" s="20"/>
-      <c r="F57" s="60"/>
-    </row>
-    <row r="58" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="67"/>
-      <c r="B58" s="20"/>
-      <c r="C58" s="6"/>
-      <c r="D58" s="68"/>
-      <c r="E58" s="62"/>
-      <c r="F58" s="63"/>
-    </row>
-    <row r="59" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="69"/>
-      <c r="B59" s="70"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="71"/>
-      <c r="E59" s="70"/>
-      <c r="F59" s="63"/>
-    </row>
-    <row r="60" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="72"/>
-      <c r="B60" s="70"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="71"/>
-      <c r="E60" s="73"/>
-      <c r="F60" s="63"/>
-    </row>
-    <row r="61" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="67"/>
-      <c r="B61" s="62"/>
-      <c r="C61" s="1"/>
-      <c r="D61" s="74"/>
-      <c r="E61" s="62"/>
-      <c r="F61" s="63"/>
-    </row>
-    <row r="62" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="75"/>
-      <c r="B62" s="62"/>
-      <c r="C62" s="1"/>
-      <c r="D62" s="74"/>
-      <c r="E62" s="62"/>
-      <c r="F62" s="63"/>
-    </row>
-    <row r="63" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="75"/>
-      <c r="B63" s="76"/>
-      <c r="C63" s="2"/>
-      <c r="D63" s="74"/>
-      <c r="E63" s="77"/>
-      <c r="F63" s="63"/>
-    </row>
-    <row r="64" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="78"/>
-      <c r="B64" s="79"/>
-      <c r="C64" s="80"/>
-      <c r="D64" s="81"/>
-      <c r="E64" s="82"/>
-      <c r="F64" s="81"/>
+    <row r="42" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A42" s="139"/>
+      <c r="B42" s="140"/>
+      <c r="C42" s="113"/>
+      <c r="D42" s="114"/>
+      <c r="E42" s="140"/>
+      <c r="F42" s="140"/>
+    </row>
+    <row r="43" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="119"/>
+      <c r="B43" s="120"/>
+      <c r="C43" s="105"/>
+      <c r="D43" s="106"/>
+      <c r="E43" s="154"/>
+      <c r="F43" s="124"/>
+    </row>
+    <row r="44" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="141"/>
+      <c r="B44" s="116"/>
+      <c r="C44" s="105"/>
+      <c r="D44" s="106"/>
+      <c r="E44" s="155"/>
+      <c r="F44" s="116"/>
+    </row>
+    <row r="45" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="119"/>
+      <c r="B45" s="116"/>
+      <c r="C45" s="105"/>
+      <c r="D45" s="106"/>
+      <c r="E45" s="120"/>
+      <c r="F45" s="124"/>
+    </row>
+    <row r="46" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="121"/>
+      <c r="B46" s="116"/>
+      <c r="C46" s="105"/>
+      <c r="D46" s="106"/>
+      <c r="E46" s="106"/>
+      <c r="F46" s="106"/>
+    </row>
+    <row r="47" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="119"/>
+      <c r="B47" s="106"/>
+      <c r="C47" s="105"/>
+      <c r="D47" s="106"/>
+      <c r="E47" s="106"/>
+      <c r="F47" s="106"/>
+    </row>
+    <row r="48" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="119"/>
+      <c r="B48" s="106"/>
+      <c r="C48" s="105"/>
+      <c r="D48" s="106"/>
+      <c r="E48" s="106"/>
+      <c r="F48" s="106"/>
+    </row>
+    <row r="49" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="119"/>
+      <c r="B49" s="106"/>
+      <c r="C49" s="105"/>
+      <c r="D49" s="106"/>
+      <c r="E49" s="106"/>
+      <c r="F49" s="106"/>
+    </row>
+    <row r="50" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="122"/>
+      <c r="B50" s="120"/>
+      <c r="C50" s="105"/>
+      <c r="D50" s="106"/>
+      <c r="E50" s="125"/>
+      <c r="F50" s="116"/>
+    </row>
+    <row r="51" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="122"/>
+      <c r="B51" s="116"/>
+      <c r="C51" s="105"/>
+      <c r="D51" s="106"/>
+      <c r="E51" s="125"/>
+      <c r="F51" s="116"/>
+    </row>
+    <row r="52" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="122"/>
+      <c r="B52" s="116"/>
+      <c r="C52" s="105"/>
+      <c r="D52" s="106"/>
+      <c r="E52" s="125"/>
+      <c r="F52" s="116"/>
+    </row>
+    <row r="53" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="122"/>
+      <c r="B53" s="116"/>
+      <c r="C53" s="105"/>
+      <c r="D53" s="106"/>
+      <c r="E53" s="125"/>
+      <c r="F53" s="116"/>
+    </row>
+    <row r="54" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="122"/>
+      <c r="B54" s="116"/>
+      <c r="C54" s="105"/>
+      <c r="D54" s="106"/>
+      <c r="E54" s="125"/>
+      <c r="F54" s="116"/>
+    </row>
+    <row r="55" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="122"/>
+      <c r="B55" s="120"/>
+      <c r="C55" s="105"/>
+      <c r="D55" s="106"/>
+      <c r="E55" s="125"/>
+      <c r="F55" s="116"/>
+    </row>
+    <row r="56" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="122"/>
+      <c r="B56" s="120"/>
+      <c r="C56" s="105"/>
+      <c r="D56" s="106"/>
+      <c r="E56" s="106"/>
+      <c r="F56" s="125"/>
+    </row>
+    <row r="57" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="122"/>
+      <c r="B57" s="106"/>
+      <c r="C57" s="105"/>
+      <c r="D57" s="106"/>
+      <c r="E57" s="106"/>
+      <c r="F57" s="116"/>
+    </row>
+    <row r="58" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="122"/>
+      <c r="B58" s="106"/>
+      <c r="C58" s="105"/>
+      <c r="D58" s="106"/>
+      <c r="E58" s="120"/>
+      <c r="F58" s="124"/>
+    </row>
+    <row r="59" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="142"/>
+      <c r="B59" s="128"/>
+      <c r="C59" s="126"/>
+      <c r="D59" s="127"/>
+      <c r="E59" s="128"/>
+      <c r="F59" s="124"/>
+    </row>
+    <row r="60" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="143"/>
+      <c r="B60" s="128"/>
+      <c r="C60" s="126"/>
+      <c r="D60" s="127"/>
+      <c r="E60" s="128"/>
+      <c r="F60" s="124"/>
+    </row>
+    <row r="61" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="122"/>
+      <c r="B61" s="120"/>
+      <c r="C61" s="105"/>
+      <c r="D61" s="129"/>
+      <c r="E61" s="120"/>
+      <c r="F61" s="124"/>
+    </row>
+    <row r="62" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="122"/>
+      <c r="B62" s="120"/>
+      <c r="C62" s="105"/>
+      <c r="D62" s="129"/>
+      <c r="E62" s="120"/>
+      <c r="F62" s="124"/>
+    </row>
+    <row r="63" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="122"/>
+      <c r="B63" s="120"/>
+      <c r="C63" s="105"/>
+      <c r="D63" s="129"/>
+      <c r="E63" s="125"/>
+      <c r="F63" s="124"/>
+    </row>
+    <row r="64" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A64" s="123"/>
+      <c r="B64" s="135"/>
+      <c r="C64" s="111"/>
+      <c r="D64" s="130"/>
+      <c r="E64" s="131"/>
+      <c r="F64" s="130"/>
     </row>
     <row r="65" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="10"/>
@@ -2293,31 +2502,31 @@
       <c r="E65" s="84"/>
       <c r="F65" s="10"/>
     </row>
-    <row r="66" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A66" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="B66" s="85"/>
+      <c r="B66" s="132"/>
       <c r="C66" s="86" t="s">
         <v>18</v>
       </c>
       <c r="D66" s="87" t="s">
         <v>19</v>
       </c>
-      <c r="E66" s="88"/>
-      <c r="F66" s="48"/>
-    </row>
-    <row r="67" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="146"/>
-      <c r="B67" s="147"/>
-      <c r="C67" s="90"/>
+      <c r="E66" s="136"/>
+      <c r="F66" s="137"/>
+    </row>
+    <row r="67" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="156"/>
+      <c r="B67" s="157"/>
+      <c r="C67" s="144"/>
       <c r="D67" s="91"/>
       <c r="E67" s="11"/>
       <c r="F67" s="92"/>
     </row>
-    <row r="68" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="93"/>
-      <c r="B68" s="74"/>
+    <row r="68" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="133"/>
+      <c r="B68" s="129"/>
       <c r="C68" s="94" t="s">
         <v>20</v>
       </c>
@@ -2325,19 +2534,19 @@
       <c r="E68" s="12"/>
       <c r="F68" s="74"/>
     </row>
-    <row r="69" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="95"/>
-      <c r="B69" s="81"/>
-      <c r="C69" s="96"/>
+    <row r="69" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="134"/>
+      <c r="B69" s="130"/>
+      <c r="C69" s="145"/>
       <c r="D69" s="10"/>
       <c r="E69" s="13"/>
       <c r="F69" s="74"/>
     </row>
-    <row r="70" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A70" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B70" s="85"/>
+      <c r="B70" s="132"/>
       <c r="C70" s="86" t="s">
         <v>43</v>
       </c>
@@ -2345,10 +2554,10 @@
       <c r="E70" s="12"/>
       <c r="F70" s="74"/>
     </row>
-    <row r="71" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="148"/>
-      <c r="B71" s="149"/>
-      <c r="C71" s="97"/>
+    <row r="71" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="158"/>
+      <c r="B71" s="159"/>
+      <c r="C71" s="146"/>
       <c r="D71" s="10"/>
       <c r="E71" s="10"/>
       <c r="F71" s="74"/>
@@ -2357,9 +2566,9 @@
       <c r="A72" s="18"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
-      <c r="D72" s="104"/>
-      <c r="E72" s="105"/>
-      <c r="F72" s="103"/>
+      <c r="D72" s="160"/>
+      <c r="E72" s="148"/>
+      <c r="F72" s="149"/>
     </row>
     <row r="73" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="98"/>
@@ -2371,11 +2580,11 @@
     </row>
     <row r="75" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A75" s="98"/>
-      <c r="D75" s="106" t="s">
+      <c r="D75" s="147" t="s">
         <v>22</v>
       </c>
-      <c r="E75" s="105"/>
-      <c r="F75" s="103"/>
+      <c r="E75" s="148"/>
+      <c r="F75" s="149"/>
     </row>
     <row r="76" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="100" t="s">
@@ -2389,13 +2598,25 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D75:F75"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="A67:B67"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="D72:F72"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D2:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A23:C23"/>
     <mergeCell ref="C39:D39"/>
     <mergeCell ref="D25:F34"/>
     <mergeCell ref="A26:C26"/>
@@ -2411,25 +2632,13 @@
     <mergeCell ref="D36:F36"/>
     <mergeCell ref="A38:B38"/>
     <mergeCell ref="D38:F38"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D2:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D75:F75"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="A67:B67"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="D72:F72"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0" bottom="0" header="0" footer="0"/>
@@ -2462,10 +2671,10 @@
       <c r="A2" s="15"/>
       <c r="B2" s="16"/>
       <c r="C2" s="17"/>
-      <c r="D2" s="107" t="s">
+      <c r="D2" s="188" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="108"/>
+      <c r="E2" s="163"/>
       <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
@@ -2474,8 +2683,8 @@
       <c r="C3" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="105"/>
-      <c r="E3" s="105"/>
+      <c r="D3" s="148"/>
+      <c r="E3" s="148"/>
       <c r="F3" s="20"/>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2484,8 +2693,8 @@
       <c r="C4" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="105"/>
-      <c r="E4" s="105"/>
+      <c r="D4" s="148"/>
+      <c r="E4" s="148"/>
       <c r="F4" s="20"/>
     </row>
     <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2494,8 +2703,8 @@
       <c r="C5" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="105"/>
-      <c r="E5" s="105"/>
+      <c r="D5" s="148"/>
+      <c r="E5" s="148"/>
       <c r="F5" s="20"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2504,20 +2713,20 @@
       <c r="C6" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="109" t="s">
+      <c r="D6" s="189" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="105"/>
+      <c r="E6" s="148"/>
       <c r="F6" s="20"/>
     </row>
     <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="18"/>
       <c r="B7" s="1"/>
       <c r="C7" s="20"/>
-      <c r="D7" s="110" t="s">
+      <c r="D7" s="190" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="105"/>
+      <c r="E7" s="148"/>
       <c r="F7" s="20"/>
     </row>
     <row r="8" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -2541,24 +2750,24 @@
       <c r="F9" s="17"/>
     </row>
     <row r="10" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="132" t="s">
+      <c r="A10" s="211" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="133"/>
-      <c r="C10" s="134"/>
-      <c r="D10" s="117"/>
-      <c r="E10" s="118"/>
-      <c r="F10" s="119"/>
+      <c r="B10" s="212"/>
+      <c r="C10" s="213"/>
+      <c r="D10" s="221"/>
+      <c r="E10" s="222"/>
+      <c r="F10" s="223"/>
     </row>
     <row r="11" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="132" t="s">
+      <c r="A11" s="211" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="133"/>
-      <c r="C11" s="134"/>
-      <c r="D11" s="117"/>
-      <c r="E11" s="118"/>
-      <c r="F11" s="119"/>
+      <c r="B11" s="212"/>
+      <c r="C11" s="213"/>
+      <c r="D11" s="221"/>
+      <c r="E11" s="222"/>
+      <c r="F11" s="223"/>
     </row>
     <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="28"/>
@@ -2594,17 +2803,17 @@
         <v>5</v>
       </c>
       <c r="C15" s="20"/>
-      <c r="D15" s="120"/>
-      <c r="E15" s="104"/>
-      <c r="F15" s="121"/>
+      <c r="D15" s="224"/>
+      <c r="E15" s="160"/>
+      <c r="F15" s="225"/>
     </row>
     <row r="16" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="33"/>
       <c r="B16" s="22"/>
       <c r="C16" s="23"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
-      <c r="F16" s="124"/>
+      <c r="D16" s="204"/>
+      <c r="E16" s="205"/>
+      <c r="F16" s="206"/>
     </row>
     <row r="17" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
@@ -2619,33 +2828,33 @@
       <c r="F17" s="17"/>
     </row>
     <row r="18" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="150"/>
-      <c r="B18" s="151"/>
-      <c r="C18" s="152"/>
-      <c r="D18" s="125"/>
-      <c r="E18" s="126"/>
-      <c r="F18" s="127"/>
+      <c r="A18" s="195"/>
+      <c r="B18" s="196"/>
+      <c r="C18" s="197"/>
+      <c r="D18" s="226"/>
+      <c r="E18" s="227"/>
+      <c r="F18" s="228"/>
     </row>
     <row r="19" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="150"/>
-      <c r="B19" s="151"/>
-      <c r="C19" s="152"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="126"/>
-      <c r="F19" s="127"/>
+      <c r="A19" s="195"/>
+      <c r="B19" s="196"/>
+      <c r="C19" s="197"/>
+      <c r="D19" s="226"/>
+      <c r="E19" s="227"/>
+      <c r="F19" s="228"/>
     </row>
     <row r="20" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="150"/>
-      <c r="B20" s="151"/>
-      <c r="C20" s="152"/>
-      <c r="D20" s="128"/>
-      <c r="E20" s="129"/>
-      <c r="F20" s="130"/>
+      <c r="A20" s="195"/>
+      <c r="B20" s="196"/>
+      <c r="C20" s="197"/>
+      <c r="D20" s="229"/>
+      <c r="E20" s="230"/>
+      <c r="F20" s="231"/>
     </row>
     <row r="21" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="150"/>
-      <c r="B21" s="151"/>
-      <c r="C21" s="152"/>
+      <c r="A21" s="195"/>
+      <c r="B21" s="196"/>
+      <c r="C21" s="197"/>
       <c r="D21" s="24" t="s">
         <v>51</v>
       </c>
@@ -2653,25 +2862,25 @@
       <c r="F21" s="17"/>
     </row>
     <row r="22" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="138"/>
-      <c r="B22" s="139"/>
-      <c r="C22" s="140"/>
+      <c r="A22" s="198"/>
+      <c r="B22" s="199"/>
+      <c r="C22" s="200"/>
       <c r="D22" s="18"/>
       <c r="E22" s="1"/>
       <c r="F22" s="20"/>
     </row>
     <row r="23" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="138"/>
-      <c r="B23" s="139"/>
-      <c r="C23" s="140"/>
+      <c r="A23" s="198"/>
+      <c r="B23" s="199"/>
+      <c r="C23" s="200"/>
       <c r="D23" s="18"/>
       <c r="E23" s="1"/>
       <c r="F23" s="20"/>
     </row>
     <row r="24" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="157"/>
-      <c r="B24" s="158"/>
-      <c r="C24" s="159"/>
+      <c r="A24" s="207"/>
+      <c r="B24" s="208"/>
+      <c r="C24" s="209"/>
       <c r="D24" s="21"/>
       <c r="E24" s="22"/>
       <c r="F24" s="23"/>
@@ -2682,67 +2891,67 @@
       </c>
       <c r="B25" s="41"/>
       <c r="C25" s="26"/>
-      <c r="D25" s="111" t="s">
+      <c r="D25" s="162" t="s">
         <v>6</v>
       </c>
-      <c r="E25" s="108"/>
-      <c r="F25" s="112"/>
+      <c r="E25" s="163"/>
+      <c r="F25" s="151"/>
     </row>
     <row r="26" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="135"/>
-      <c r="B26" s="136"/>
-      <c r="C26" s="137"/>
-      <c r="D26" s="113"/>
-      <c r="E26" s="105"/>
-      <c r="F26" s="103"/>
+      <c r="A26" s="214"/>
+      <c r="B26" s="215"/>
+      <c r="C26" s="216"/>
+      <c r="D26" s="164"/>
+      <c r="E26" s="148"/>
+      <c r="F26" s="149"/>
     </row>
     <row r="27" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="138"/>
-      <c r="B27" s="139"/>
-      <c r="C27" s="140"/>
-      <c r="D27" s="113"/>
-      <c r="E27" s="105"/>
-      <c r="F27" s="103"/>
+      <c r="A27" s="198"/>
+      <c r="B27" s="199"/>
+      <c r="C27" s="200"/>
+      <c r="D27" s="164"/>
+      <c r="E27" s="148"/>
+      <c r="F27" s="149"/>
     </row>
     <row r="28" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="138"/>
-      <c r="B28" s="139"/>
-      <c r="C28" s="140"/>
-      <c r="D28" s="113"/>
-      <c r="E28" s="105"/>
-      <c r="F28" s="103"/>
+      <c r="A28" s="198"/>
+      <c r="B28" s="199"/>
+      <c r="C28" s="200"/>
+      <c r="D28" s="164"/>
+      <c r="E28" s="148"/>
+      <c r="F28" s="149"/>
     </row>
     <row r="29" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="138"/>
-      <c r="B29" s="139"/>
-      <c r="C29" s="140"/>
-      <c r="D29" s="113"/>
-      <c r="E29" s="105"/>
-      <c r="F29" s="103"/>
+      <c r="A29" s="198"/>
+      <c r="B29" s="199"/>
+      <c r="C29" s="200"/>
+      <c r="D29" s="164"/>
+      <c r="E29" s="148"/>
+      <c r="F29" s="149"/>
     </row>
     <row r="30" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="138"/>
-      <c r="B30" s="139"/>
-      <c r="C30" s="140"/>
-      <c r="D30" s="113"/>
-      <c r="E30" s="105"/>
-      <c r="F30" s="103"/>
+      <c r="A30" s="198"/>
+      <c r="B30" s="199"/>
+      <c r="C30" s="200"/>
+      <c r="D30" s="164"/>
+      <c r="E30" s="148"/>
+      <c r="F30" s="149"/>
     </row>
     <row r="31" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="138"/>
-      <c r="B31" s="139"/>
-      <c r="C31" s="140"/>
-      <c r="D31" s="113"/>
-      <c r="E31" s="105"/>
-      <c r="F31" s="103"/>
+      <c r="A31" s="198"/>
+      <c r="B31" s="199"/>
+      <c r="C31" s="200"/>
+      <c r="D31" s="164"/>
+      <c r="E31" s="148"/>
+      <c r="F31" s="149"/>
     </row>
     <row r="32" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="141"/>
-      <c r="B32" s="142"/>
-      <c r="C32" s="143"/>
-      <c r="D32" s="113"/>
-      <c r="E32" s="105"/>
-      <c r="F32" s="103"/>
+      <c r="A32" s="217"/>
+      <c r="B32" s="218"/>
+      <c r="C32" s="219"/>
+      <c r="D32" s="164"/>
+      <c r="E32" s="148"/>
+      <c r="F32" s="149"/>
     </row>
     <row r="33" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="24" t="s">
@@ -2752,23 +2961,23 @@
       <c r="C33" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="D33" s="113"/>
-      <c r="E33" s="105"/>
-      <c r="F33" s="103"/>
+      <c r="D33" s="164"/>
+      <c r="E33" s="148"/>
+      <c r="F33" s="149"/>
     </row>
     <row r="34" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="144"/>
-      <c r="B34" s="145"/>
+      <c r="A34" s="201"/>
+      <c r="B34" s="202"/>
       <c r="C34" s="47"/>
-      <c r="D34" s="114"/>
-      <c r="E34" s="115"/>
-      <c r="F34" s="116"/>
+      <c r="D34" s="165"/>
+      <c r="E34" s="166"/>
+      <c r="F34" s="153"/>
     </row>
     <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="131" t="s">
+      <c r="A35" s="175" t="s">
         <v>47</v>
       </c>
-      <c r="B35" s="112"/>
+      <c r="B35" s="151"/>
       <c r="C35" s="46" t="s">
         <v>48</v>
       </c>
@@ -2779,12 +2988,12 @@
       <c r="F35" s="17"/>
     </row>
     <row r="36" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="160"/>
-      <c r="B36" s="116"/>
+      <c r="A36" s="210"/>
+      <c r="B36" s="153"/>
       <c r="C36" s="47"/>
-      <c r="D36" s="122"/>
-      <c r="E36" s="123"/>
-      <c r="F36" s="124"/>
+      <c r="D36" s="204"/>
+      <c r="E36" s="205"/>
+      <c r="F36" s="206"/>
     </row>
     <row r="37" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="24" t="s">
@@ -2801,18 +3010,18 @@
       <c r="F37" s="17"/>
     </row>
     <row r="38" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="144"/>
-      <c r="B38" s="145"/>
+      <c r="A38" s="201"/>
+      <c r="B38" s="202"/>
       <c r="C38" s="49"/>
-      <c r="D38" s="144"/>
-      <c r="E38" s="156"/>
-      <c r="F38" s="145"/>
+      <c r="D38" s="201"/>
+      <c r="E38" s="203"/>
+      <c r="F38" s="202"/>
     </row>
     <row r="39" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
-      <c r="C39" s="153"/>
-      <c r="D39" s="105"/>
+      <c r="C39" s="161"/>
+      <c r="D39" s="148"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
     </row>
@@ -2823,10 +3032,10 @@
       <c r="B40" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="154" t="s">
+      <c r="C40" s="150" t="s">
         <v>9</v>
       </c>
-      <c r="D40" s="112"/>
+      <c r="D40" s="151"/>
       <c r="E40" s="50" t="s">
         <v>10</v>
       </c>
@@ -2839,8 +3048,8 @@
         <v>7</v>
       </c>
       <c r="B41" s="51"/>
-      <c r="C41" s="155"/>
-      <c r="D41" s="116"/>
+      <c r="C41" s="152"/>
+      <c r="D41" s="153"/>
       <c r="E41" s="51" t="s">
         <v>59</v>
       </c>
@@ -2861,7 +3070,7 @@
       <c r="B43" s="56"/>
       <c r="C43" s="1"/>
       <c r="D43" s="57"/>
-      <c r="E43" s="102"/>
+      <c r="E43" s="220"/>
       <c r="F43" s="58"/>
     </row>
     <row r="44" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2869,7 +3078,7 @@
       <c r="B44" s="60"/>
       <c r="C44" s="1"/>
       <c r="D44" s="20"/>
-      <c r="E44" s="103"/>
+      <c r="E44" s="149"/>
       <c r="F44" s="60"/>
     </row>
     <row r="45" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3055,8 +3264,8 @@
       <c r="F66" s="48"/>
     </row>
     <row r="67" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="146"/>
-      <c r="B67" s="147"/>
+      <c r="A67" s="191"/>
+      <c r="B67" s="192"/>
       <c r="C67" s="90"/>
       <c r="D67" s="91"/>
       <c r="E67" s="11"/>
@@ -3093,8 +3302,8 @@
       <c r="F70" s="74"/>
     </row>
     <row r="71" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="148"/>
-      <c r="B71" s="149"/>
+      <c r="A71" s="193"/>
+      <c r="B71" s="194"/>
       <c r="C71" s="97"/>
       <c r="D71" s="10"/>
       <c r="E71" s="10"/>
@@ -3104,9 +3313,9 @@
       <c r="A72" s="18"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
-      <c r="D72" s="104"/>
-      <c r="E72" s="105"/>
-      <c r="F72" s="103"/>
+      <c r="D72" s="160"/>
+      <c r="E72" s="148"/>
+      <c r="F72" s="149"/>
     </row>
     <row r="73" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="98"/>
@@ -3118,11 +3327,11 @@
     </row>
     <row r="75" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A75" s="98"/>
-      <c r="D75" s="106" t="s">
+      <c r="D75" s="147" t="s">
         <v>22</v>
       </c>
-      <c r="E75" s="105"/>
-      <c r="F75" s="103"/>
+      <c r="E75" s="148"/>
+      <c r="F75" s="149"/>
     </row>
     <row r="76" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="100" t="s">
@@ -3136,6 +3345,31 @@
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="D72:F72"/>
+    <mergeCell ref="D75:F75"/>
+    <mergeCell ref="D2:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D25:F34"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A34:B34"/>
     <mergeCell ref="A67:B67"/>
     <mergeCell ref="A71:B71"/>
     <mergeCell ref="A18:C18"/>
@@ -3152,31 +3386,6 @@
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="D72:F72"/>
-    <mergeCell ref="D75:F75"/>
-    <mergeCell ref="D2:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D25:F34"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:F20"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0" bottom="0" header="0" footer="0"/>
@@ -3206,10 +3415,10 @@
       <c r="A2" s="15"/>
       <c r="B2" s="16"/>
       <c r="C2" s="17"/>
-      <c r="D2" s="107" t="s">
+      <c r="D2" s="188" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="108"/>
+      <c r="E2" s="163"/>
       <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
@@ -3218,8 +3427,8 @@
       <c r="C3" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="105"/>
-      <c r="E3" s="105"/>
+      <c r="D3" s="148"/>
+      <c r="E3" s="148"/>
       <c r="F3" s="20"/>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3228,8 +3437,8 @@
       <c r="C4" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="105"/>
-      <c r="E4" s="105"/>
+      <c r="D4" s="148"/>
+      <c r="E4" s="148"/>
       <c r="F4" s="20"/>
     </row>
     <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3238,8 +3447,8 @@
       <c r="C5" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="105"/>
-      <c r="E5" s="105"/>
+      <c r="D5" s="148"/>
+      <c r="E5" s="148"/>
       <c r="F5" s="20"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3248,20 +3457,20 @@
       <c r="C6" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="109" t="s">
+      <c r="D6" s="189" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="105"/>
+      <c r="E6" s="148"/>
       <c r="F6" s="20"/>
     </row>
     <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="18"/>
       <c r="B7" s="1"/>
       <c r="C7" s="20"/>
-      <c r="D7" s="110" t="s">
+      <c r="D7" s="190" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="105"/>
+      <c r="E7" s="148"/>
       <c r="F7" s="20"/>
     </row>
     <row r="8" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3422,67 +3631,67 @@
       </c>
       <c r="B25" s="41"/>
       <c r="C25" s="26"/>
-      <c r="D25" s="111" t="s">
+      <c r="D25" s="162" t="s">
         <v>6</v>
       </c>
-      <c r="E25" s="108"/>
-      <c r="F25" s="112"/>
+      <c r="E25" s="163"/>
+      <c r="F25" s="151"/>
     </row>
     <row r="26" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="42"/>
       <c r="B26" s="7"/>
       <c r="C26" s="43"/>
-      <c r="D26" s="113"/>
-      <c r="E26" s="105"/>
-      <c r="F26" s="103"/>
+      <c r="D26" s="164"/>
+      <c r="E26" s="148"/>
+      <c r="F26" s="149"/>
     </row>
     <row r="27" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="38"/>
       <c r="B27" s="6"/>
       <c r="C27" s="20"/>
-      <c r="D27" s="113"/>
-      <c r="E27" s="105"/>
-      <c r="F27" s="103"/>
+      <c r="D27" s="164"/>
+      <c r="E27" s="148"/>
+      <c r="F27" s="149"/>
     </row>
     <row r="28" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="38"/>
       <c r="B28" s="6"/>
       <c r="C28" s="20"/>
-      <c r="D28" s="113"/>
-      <c r="E28" s="105"/>
-      <c r="F28" s="103"/>
+      <c r="D28" s="164"/>
+      <c r="E28" s="148"/>
+      <c r="F28" s="149"/>
     </row>
     <row r="29" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="38"/>
       <c r="B29" s="6"/>
       <c r="C29" s="20"/>
-      <c r="D29" s="113"/>
-      <c r="E29" s="105"/>
-      <c r="F29" s="103"/>
+      <c r="D29" s="164"/>
+      <c r="E29" s="148"/>
+      <c r="F29" s="149"/>
     </row>
     <row r="30" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="38"/>
       <c r="B30" s="6"/>
       <c r="C30" s="20"/>
-      <c r="D30" s="113"/>
-      <c r="E30" s="105"/>
-      <c r="F30" s="103"/>
+      <c r="D30" s="164"/>
+      <c r="E30" s="148"/>
+      <c r="F30" s="149"/>
     </row>
     <row r="31" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="38"/>
       <c r="B31" s="6"/>
       <c r="C31" s="20"/>
-      <c r="D31" s="113"/>
-      <c r="E31" s="105"/>
-      <c r="F31" s="103"/>
+      <c r="D31" s="164"/>
+      <c r="E31" s="148"/>
+      <c r="F31" s="149"/>
     </row>
     <row r="32" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="44"/>
       <c r="B32" s="22"/>
       <c r="C32" s="45"/>
-      <c r="D32" s="113"/>
-      <c r="E32" s="105"/>
-      <c r="F32" s="103"/>
+      <c r="D32" s="164"/>
+      <c r="E32" s="148"/>
+      <c r="F32" s="149"/>
     </row>
     <row r="33" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="24" t="s">
@@ -3492,23 +3701,23 @@
       <c r="C33" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="D33" s="113"/>
-      <c r="E33" s="105"/>
-      <c r="F33" s="103"/>
+      <c r="D33" s="164"/>
+      <c r="E33" s="148"/>
+      <c r="F33" s="149"/>
     </row>
     <row r="34" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="33"/>
       <c r="B34" s="22"/>
       <c r="C34" s="47"/>
-      <c r="D34" s="114"/>
-      <c r="E34" s="115"/>
-      <c r="F34" s="116"/>
+      <c r="D34" s="165"/>
+      <c r="E34" s="166"/>
+      <c r="F34" s="153"/>
     </row>
     <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="131" t="s">
+      <c r="A35" s="175" t="s">
         <v>47</v>
       </c>
-      <c r="B35" s="112"/>
+      <c r="B35" s="151"/>
       <c r="C35" s="46" t="s">
         <v>48</v>
       </c>
@@ -3519,8 +3728,8 @@
       <c r="F35" s="17"/>
     </row>
     <row r="36" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="160"/>
-      <c r="B36" s="116"/>
+      <c r="A36" s="210"/>
+      <c r="B36" s="153"/>
       <c r="C36" s="47"/>
       <c r="D36" s="21"/>
       <c r="E36" s="22"/>
@@ -3551,8 +3760,8 @@
     <row r="39" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
-      <c r="C39" s="153"/>
-      <c r="D39" s="105"/>
+      <c r="C39" s="161"/>
+      <c r="D39" s="148"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
     </row>
@@ -3563,10 +3772,10 @@
       <c r="B40" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="154" t="s">
+      <c r="C40" s="150" t="s">
         <v>9</v>
       </c>
-      <c r="D40" s="112"/>
+      <c r="D40" s="151"/>
       <c r="E40" s="50" t="s">
         <v>10</v>
       </c>
@@ -3579,8 +3788,8 @@
         <v>7</v>
       </c>
       <c r="B41" s="51"/>
-      <c r="C41" s="155"/>
-      <c r="D41" s="116"/>
+      <c r="C41" s="152"/>
+      <c r="D41" s="153"/>
       <c r="E41" s="51" t="s">
         <v>59</v>
       </c>
@@ -3601,7 +3810,7 @@
       <c r="B43" s="56"/>
       <c r="C43" s="1"/>
       <c r="D43" s="57"/>
-      <c r="E43" s="102"/>
+      <c r="E43" s="220"/>
       <c r="F43" s="58"/>
     </row>
     <row r="44" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3609,7 +3818,7 @@
       <c r="B44" s="60"/>
       <c r="C44" s="1"/>
       <c r="D44" s="20"/>
-      <c r="E44" s="103"/>
+      <c r="E44" s="149"/>
       <c r="F44" s="60"/>
     </row>
     <row r="45" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3844,9 +4053,9 @@
       <c r="A72" s="18"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
-      <c r="D72" s="104"/>
-      <c r="E72" s="105"/>
-      <c r="F72" s="103"/>
+      <c r="D72" s="160"/>
+      <c r="E72" s="148"/>
+      <c r="F72" s="149"/>
     </row>
     <row r="73" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="98"/>
@@ -3858,11 +4067,11 @@
     </row>
     <row r="75" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A75" s="98"/>
-      <c r="D75" s="106" t="s">
+      <c r="D75" s="147" t="s">
         <v>22</v>
       </c>
-      <c r="E75" s="105"/>
-      <c r="F75" s="103"/>
+      <c r="E75" s="148"/>
+      <c r="F75" s="149"/>
     </row>
     <row r="76" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="100" t="s">
@@ -3922,10 +4131,10 @@
       <c r="B7" s="15"/>
       <c r="C7" s="16"/>
       <c r="D7" s="17"/>
-      <c r="E7" s="107" t="s">
+      <c r="E7" s="188" t="s">
         <v>0</v>
       </c>
-      <c r="F7" s="108"/>
+      <c r="F7" s="163"/>
       <c r="G7" s="17"/>
     </row>
     <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
@@ -3935,8 +4144,8 @@
       <c r="D8" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="105"/>
-      <c r="F8" s="105"/>
+      <c r="E8" s="148"/>
+      <c r="F8" s="148"/>
       <c r="G8" s="20"/>
     </row>
     <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3946,8 +4155,8 @@
       <c r="D9" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="105"/>
-      <c r="F9" s="105"/>
+      <c r="E9" s="148"/>
+      <c r="F9" s="148"/>
       <c r="G9" s="20"/>
     </row>
     <row r="10" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3957,8 +4166,8 @@
       <c r="D10" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="105"/>
-      <c r="F10" s="105"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="148"/>
       <c r="G10" s="20"/>
     </row>
     <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3968,10 +4177,10 @@
       <c r="D11" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="109" t="s">
+      <c r="E11" s="189" t="s">
         <v>1</v>
       </c>
-      <c r="F11" s="105"/>
+      <c r="F11" s="148"/>
       <c r="G11" s="20"/>
     </row>
     <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
@@ -3979,10 +4188,10 @@
       <c r="B12" s="18"/>
       <c r="C12" s="1"/>
       <c r="D12" s="20"/>
-      <c r="E12" s="110" t="s">
+      <c r="E12" s="190" t="s">
         <v>42</v>
       </c>
-      <c r="F12" s="105"/>
+      <c r="F12" s="148"/>
       <c r="G12" s="20"/>
     </row>
     <row r="13" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -4161,74 +4370,74 @@
       </c>
       <c r="C30" s="41"/>
       <c r="D30" s="26"/>
-      <c r="E30" s="111" t="s">
+      <c r="E30" s="162" t="s">
         <v>6</v>
       </c>
-      <c r="F30" s="108"/>
-      <c r="G30" s="112"/>
+      <c r="F30" s="163"/>
+      <c r="G30" s="151"/>
     </row>
     <row r="31" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="42"/>
       <c r="C31" s="7"/>
       <c r="D31" s="43"/>
-      <c r="E31" s="113"/>
-      <c r="F31" s="105"/>
-      <c r="G31" s="103"/>
+      <c r="E31" s="164"/>
+      <c r="F31" s="148"/>
+      <c r="G31" s="149"/>
     </row>
     <row r="32" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="38"/>
       <c r="C32" s="6"/>
       <c r="D32" s="20"/>
-      <c r="E32" s="113"/>
-      <c r="F32" s="105"/>
-      <c r="G32" s="103"/>
+      <c r="E32" s="164"/>
+      <c r="F32" s="148"/>
+      <c r="G32" s="149"/>
     </row>
     <row r="33" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="38"/>
       <c r="C33" s="6"/>
       <c r="D33" s="20"/>
-      <c r="E33" s="113"/>
-      <c r="F33" s="105"/>
-      <c r="G33" s="103"/>
+      <c r="E33" s="164"/>
+      <c r="F33" s="148"/>
+      <c r="G33" s="149"/>
     </row>
     <row r="34" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="38"/>
       <c r="C34" s="6"/>
       <c r="D34" s="20"/>
-      <c r="E34" s="113"/>
-      <c r="F34" s="105"/>
-      <c r="G34" s="103"/>
+      <c r="E34" s="164"/>
+      <c r="F34" s="148"/>
+      <c r="G34" s="149"/>
     </row>
     <row r="35" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="38"/>
       <c r="C35" s="6"/>
       <c r="D35" s="20"/>
-      <c r="E35" s="113"/>
-      <c r="F35" s="105"/>
-      <c r="G35" s="103"/>
+      <c r="E35" s="164"/>
+      <c r="F35" s="148"/>
+      <c r="G35" s="149"/>
     </row>
     <row r="36" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="38"/>
       <c r="C36" s="6"/>
       <c r="D36" s="20"/>
-      <c r="E36" s="113"/>
-      <c r="F36" s="105"/>
-      <c r="G36" s="103"/>
+      <c r="E36" s="164"/>
+      <c r="F36" s="148"/>
+      <c r="G36" s="149"/>
     </row>
     <row r="37" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="44"/>
       <c r="C37" s="22"/>
       <c r="D37" s="45"/>
-      <c r="E37" s="113"/>
-      <c r="F37" s="105"/>
-      <c r="G37" s="103"/>
+      <c r="E37" s="164"/>
+      <c r="F37" s="148"/>
+      <c r="G37" s="149"/>
     </row>
     <row r="38" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
@@ -4237,25 +4446,25 @@
       </c>
       <c r="C38" s="16"/>
       <c r="D38" s="17"/>
-      <c r="E38" s="113"/>
-      <c r="F38" s="105"/>
-      <c r="G38" s="103"/>
+      <c r="E38" s="164"/>
+      <c r="F38" s="148"/>
+      <c r="G38" s="149"/>
     </row>
     <row r="39" spans="1:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="33"/>
       <c r="C39" s="22"/>
       <c r="D39" s="40"/>
-      <c r="E39" s="114"/>
-      <c r="F39" s="115"/>
-      <c r="G39" s="116"/>
+      <c r="E39" s="165"/>
+      <c r="F39" s="166"/>
+      <c r="G39" s="153"/>
     </row>
     <row r="40" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="131" t="s">
+      <c r="B40" s="175" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="112"/>
+      <c r="C40" s="151"/>
       <c r="D40" s="46" t="s">
         <v>36</v>
       </c>
@@ -4267,8 +4476,8 @@
     </row>
     <row r="41" spans="1:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
-      <c r="B41" s="160"/>
-      <c r="C41" s="116"/>
+      <c r="B41" s="210"/>
+      <c r="C41" s="153"/>
       <c r="D41" s="47"/>
       <c r="E41" s="21"/>
       <c r="F41" s="22"/>
@@ -4302,8 +4511,8 @@
       <c r="A44" s="1"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
-      <c r="D44" s="153"/>
-      <c r="E44" s="105"/>
+      <c r="D44" s="161"/>
+      <c r="E44" s="148"/>
       <c r="F44" s="7"/>
       <c r="G44" s="7"/>
     </row>
@@ -4315,10 +4524,10 @@
       <c r="C45" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="D45" s="154" t="s">
+      <c r="D45" s="150" t="s">
         <v>9</v>
       </c>
-      <c r="E45" s="112"/>
+      <c r="E45" s="151"/>
       <c r="F45" s="50" t="s">
         <v>10</v>
       </c>
@@ -4334,10 +4543,10 @@
       <c r="C46" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="D46" s="155" t="s">
+      <c r="D46" s="152" t="s">
         <v>14</v>
       </c>
-      <c r="E46" s="116"/>
+      <c r="E46" s="153"/>
       <c r="F46" s="51" t="s">
         <v>15</v>
       </c>
@@ -4360,7 +4569,7 @@
       <c r="C48" s="56"/>
       <c r="D48" s="1"/>
       <c r="E48" s="57"/>
-      <c r="F48" s="102"/>
+      <c r="F48" s="220"/>
       <c r="G48" s="58"/>
     </row>
     <row r="49" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4369,7 +4578,7 @@
       <c r="C49" s="60"/>
       <c r="D49" s="1"/>
       <c r="E49" s="20"/>
-      <c r="F49" s="103"/>
+      <c r="F49" s="149"/>
       <c r="G49" s="60"/>
     </row>
     <row r="50" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4632,9 +4841,9 @@
       <c r="B77" s="18"/>
       <c r="C77" s="1"/>
       <c r="D77" s="1"/>
-      <c r="E77" s="104"/>
-      <c r="F77" s="105"/>
-      <c r="G77" s="103"/>
+      <c r="E77" s="160"/>
+      <c r="F77" s="148"/>
+      <c r="G77" s="149"/>
     </row>
     <row r="78" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B78" s="98"/>
@@ -4646,11 +4855,11 @@
     </row>
     <row r="80" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B80" s="98"/>
-      <c r="E80" s="106" t="s">
+      <c r="E80" s="147" t="s">
         <v>22</v>
       </c>
-      <c r="F80" s="105"/>
-      <c r="G80" s="103"/>
+      <c r="F80" s="148"/>
+      <c r="G80" s="149"/>
     </row>
     <row r="81" spans="2:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B81" s="100" t="s">

</xml_diff>

<commit_message>
Modificaciones en plantilla para ajustar el forwarding
</commit_message>
<xml_diff>
--- a/plantillas/template.xlsx
+++ b/plantillas/template.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/02a88c3211e78dcc/Escritorio/Iacc/proyectos/SDW_V2/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="255" documentId="13_ncr:1_{31C7B298-62C6-4CC3-9913-170867C88746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC787503-3612-4A83-8CBD-4FBAB924B17F}"/>
+  <xr:revisionPtr revIDLastSave="271" documentId="13_ncr:1_{31C7B298-62C6-4CC3-9913-170867C88746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65576B22-4F70-4E1E-AC49-3B0DA91D867D}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ORIGINAL" sheetId="9" r:id="rId1"/>
-    <sheet name="COPY NO NEGOCIABLE" sheetId="4" r:id="rId2"/>
+    <sheet name="ORIGINAL" sheetId="10" r:id="rId1"/>
+    <sheet name="COPY NO NEGOCIABLE" sheetId="9" r:id="rId2"/>
     <sheet name="COPY NO NEGOCIABLE 1" sheetId="8" state="hidden" r:id="rId3"/>
     <sheet name="ingles espanol" sheetId="7" state="hidden" r:id="rId4"/>
   </sheets>
@@ -649,7 +649,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="232">
+  <cellXfs count="196">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -913,19 +913,108 @@
     <xf numFmtId="49" fontId="38" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="34" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -945,207 +1034,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1188,6 +1080,158 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1038225</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4667250" cy="38100"/>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="2" name="Shape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AAD7965-AD1F-4956-8E3F-F7051BC31731}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="7667625" y="17297400"/>
+          <a:ext cx="4667250" cy="38100"/>
+          <a:chOff x="3012375" y="3780000"/>
+          <a:chExt cx="4667250" cy="0"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="3" name="Shape 4">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6542708B-04B8-82E4-0C90-23F8BA67DC02}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3012375" y="3780000"/>
+            <a:ext cx="4667250" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="straightConnector1">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="12700" cap="flat" cmpd="sng">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+            <a:miter lim="800000"/>
+            <a:headEnd type="none" w="sm" len="sm"/>
+            <a:tailEnd type="none" w="sm" len="sm"/>
+          </a:ln>
+        </xdr:spPr>
+      </xdr:cxnSp>
+    </xdr:grpSp>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2771775" cy="1200150"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="image1.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9CA3B218-F030-48DD-A081-12658D04E33B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:srcRect l="4652" t="7936" r="4264" b="7936"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="266700" y="200025"/>
+          <a:ext cx="2771775" cy="1200150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2028824</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>57595</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1981199</xdr:colOff>
+      <xdr:row>72</xdr:row>
+      <xdr:rowOff>139077</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagen 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E3E646F-04F2-47FF-A3F9-66853749D5CC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8658224" y="15602395"/>
+          <a:ext cx="2143125" cy="1529282"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
@@ -1308,158 +1352,6 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A717E887-7D7F-46FD-885C-46D5D7C2B332}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8658224" y="14916595"/>
-          <a:ext cx="2143125" cy="1529282"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1038225</xdr:colOff>
-      <xdr:row>73</xdr:row>
-      <xdr:rowOff>104775</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="4667250" cy="38100"/>
-    <xdr:grpSp>
-      <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="2" name="Shape 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGrpSpPr/>
-      </xdr:nvGrpSpPr>
-      <xdr:grpSpPr>
-        <a:xfrm>
-          <a:off x="7667625" y="16554450"/>
-          <a:ext cx="4667250" cy="38100"/>
-          <a:chOff x="3012375" y="3780000"/>
-          <a:chExt cx="4667250" cy="0"/>
-        </a:xfrm>
-      </xdr:grpSpPr>
-      <xdr:cxnSp macro="">
-        <xdr:nvCxnSpPr>
-          <xdr:cNvPr id="4" name="Shape 4">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000004000000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvCxnSpPr/>
-        </xdr:nvCxnSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="3012375" y="3780000"/>
-            <a:ext cx="4667250" cy="0"/>
-          </a:xfrm>
-          <a:prstGeom prst="straightConnector1">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln w="12700" cap="flat" cmpd="sng">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-            <a:miter lim="800000"/>
-            <a:headEnd type="none" w="sm" len="sm"/>
-            <a:tailEnd type="none" w="sm" len="sm"/>
-          </a:ln>
-        </xdr:spPr>
-      </xdr:cxnSp>
-    </xdr:grpSp>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>266700</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2771775" cy="1200150"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="image1.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000003000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:srcRect l="4652" t="7936" r="4264" b="7936"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="266700" y="200025"/>
-          <a:ext cx="2771775" cy="1200150"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>2028824</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>57595</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>1981199</xdr:colOff>
-      <xdr:row>72</xdr:row>
-      <xdr:rowOff>196227</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Imagen 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9748DB04-A2C0-4787-BB1C-E041F494B713}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1901,6 +1793,752 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBC52D04-E9C6-4482-9560-09AA58C2138C}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F76"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.75" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="44.25" customWidth="1"/>
+    <col min="4" max="4" width="28.75" customWidth="1"/>
+    <col min="5" max="6" width="27.25" customWidth="1"/>
+    <col min="7" max="25" width="10.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="14"/>
+      <c r="F1" s="14"/>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="15"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="150" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="151"/>
+      <c r="F2" s="17"/>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="18"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="152"/>
+      <c r="E3" s="152"/>
+      <c r="F3" s="20"/>
+    </row>
+    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="18"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="152"/>
+      <c r="E4" s="152"/>
+      <c r="F4" s="20"/>
+    </row>
+    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="18"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="152"/>
+      <c r="E5" s="152"/>
+      <c r="F5" s="20"/>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="18"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="153" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" s="152"/>
+      <c r="F6" s="20"/>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="18"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="154" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" s="152"/>
+      <c r="F7" s="20"/>
+    </row>
+    <row r="8" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="21"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="23"/>
+    </row>
+    <row r="9" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A9" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="25"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="113"/>
+      <c r="F9" s="114"/>
+    </row>
+    <row r="10" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="147" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="148"/>
+      <c r="C10" s="149"/>
+      <c r="D10" s="147"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="149"/>
+    </row>
+    <row r="11" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="147" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" s="148"/>
+      <c r="C11" s="149"/>
+      <c r="D11" s="147"/>
+      <c r="E11" s="148"/>
+      <c r="F11" s="149"/>
+    </row>
+    <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="104"/>
+      <c r="B12" s="105"/>
+      <c r="C12" s="106"/>
+      <c r="D12" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" s="105"/>
+      <c r="F12" s="106"/>
+    </row>
+    <row r="13" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="107"/>
+      <c r="B13" s="105"/>
+      <c r="C13" s="106"/>
+      <c r="D13" s="115"/>
+      <c r="E13" s="111"/>
+      <c r="F13" s="112"/>
+    </row>
+    <row r="14" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="104"/>
+      <c r="B14" s="105"/>
+      <c r="C14" s="106"/>
+      <c r="D14" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" s="113"/>
+      <c r="F14" s="114"/>
+    </row>
+    <row r="15" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="108"/>
+      <c r="B15" s="109" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="106"/>
+      <c r="D15" s="158"/>
+      <c r="E15" s="159"/>
+      <c r="F15" s="160"/>
+    </row>
+    <row r="16" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="110"/>
+      <c r="B16" s="111"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="161"/>
+      <c r="E16" s="162"/>
+      <c r="F16" s="163"/>
+    </row>
+    <row r="17" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A17" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="25"/>
+      <c r="C17" s="118"/>
+      <c r="D17" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="E17" s="113"/>
+      <c r="F17" s="114"/>
+    </row>
+    <row r="18" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="164"/>
+      <c r="B18" s="165"/>
+      <c r="C18" s="166"/>
+      <c r="D18" s="170"/>
+      <c r="E18" s="171"/>
+      <c r="F18" s="172"/>
+    </row>
+    <row r="19" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="164"/>
+      <c r="B19" s="165"/>
+      <c r="C19" s="166"/>
+      <c r="D19" s="170"/>
+      <c r="E19" s="171"/>
+      <c r="F19" s="172"/>
+    </row>
+    <row r="20" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="164"/>
+      <c r="B20" s="165"/>
+      <c r="C20" s="166"/>
+      <c r="D20" s="167"/>
+      <c r="E20" s="168"/>
+      <c r="F20" s="169"/>
+    </row>
+    <row r="21" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="164"/>
+      <c r="B21" s="165"/>
+      <c r="C21" s="166"/>
+      <c r="D21" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="E21" s="113"/>
+      <c r="F21" s="114"/>
+    </row>
+    <row r="22" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="170"/>
+      <c r="B22" s="171"/>
+      <c r="C22" s="172"/>
+      <c r="D22" s="117"/>
+      <c r="E22" s="105"/>
+      <c r="F22" s="106"/>
+    </row>
+    <row r="23" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="170"/>
+      <c r="B23" s="171"/>
+      <c r="C23" s="172"/>
+      <c r="D23" s="117"/>
+      <c r="E23" s="105"/>
+      <c r="F23" s="106"/>
+    </row>
+    <row r="24" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="155"/>
+      <c r="B24" s="156"/>
+      <c r="C24" s="157"/>
+      <c r="D24" s="115"/>
+      <c r="E24" s="111"/>
+      <c r="F24" s="112"/>
+    </row>
+    <row r="25" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A25" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" s="113"/>
+      <c r="C25" s="118"/>
+      <c r="D25" s="174" t="s">
+        <v>6</v>
+      </c>
+      <c r="E25" s="151"/>
+      <c r="F25" s="175"/>
+    </row>
+    <row r="26" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="170"/>
+      <c r="B26" s="171"/>
+      <c r="C26" s="172"/>
+      <c r="D26" s="176"/>
+      <c r="E26" s="152"/>
+      <c r="F26" s="177"/>
+    </row>
+    <row r="27" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="170"/>
+      <c r="B27" s="171"/>
+      <c r="C27" s="172"/>
+      <c r="D27" s="176"/>
+      <c r="E27" s="152"/>
+      <c r="F27" s="177"/>
+    </row>
+    <row r="28" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="170"/>
+      <c r="B28" s="171"/>
+      <c r="C28" s="172"/>
+      <c r="D28" s="176"/>
+      <c r="E28" s="152"/>
+      <c r="F28" s="177"/>
+    </row>
+    <row r="29" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="170"/>
+      <c r="B29" s="171"/>
+      <c r="C29" s="172"/>
+      <c r="D29" s="176"/>
+      <c r="E29" s="152"/>
+      <c r="F29" s="177"/>
+    </row>
+    <row r="30" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="170"/>
+      <c r="B30" s="171"/>
+      <c r="C30" s="172"/>
+      <c r="D30" s="176"/>
+      <c r="E30" s="152"/>
+      <c r="F30" s="177"/>
+    </row>
+    <row r="31" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="170"/>
+      <c r="B31" s="171"/>
+      <c r="C31" s="172"/>
+      <c r="D31" s="176"/>
+      <c r="E31" s="152"/>
+      <c r="F31" s="177"/>
+    </row>
+    <row r="32" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="167"/>
+      <c r="B32" s="168"/>
+      <c r="C32" s="169"/>
+      <c r="D32" s="176"/>
+      <c r="E32" s="152"/>
+      <c r="F32" s="177"/>
+    </row>
+    <row r="33" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A33" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="113"/>
+      <c r="C33" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="D33" s="176"/>
+      <c r="E33" s="152"/>
+      <c r="F33" s="177"/>
+    </row>
+    <row r="34" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="161"/>
+      <c r="B34" s="163"/>
+      <c r="C34" s="123"/>
+      <c r="D34" s="178"/>
+      <c r="E34" s="179"/>
+      <c r="F34" s="180"/>
+    </row>
+    <row r="35" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A35" s="181" t="s">
+        <v>47</v>
+      </c>
+      <c r="B35" s="175"/>
+      <c r="C35" s="46" t="s">
+        <v>48</v>
+      </c>
+      <c r="D35" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="E35" s="16"/>
+      <c r="F35" s="114"/>
+    </row>
+    <row r="36" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="182"/>
+      <c r="B36" s="183"/>
+      <c r="C36" s="103"/>
+      <c r="D36" s="161"/>
+      <c r="E36" s="162"/>
+      <c r="F36" s="163"/>
+    </row>
+    <row r="37" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A37" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B37" s="102"/>
+      <c r="C37" s="46" t="s">
+        <v>45</v>
+      </c>
+      <c r="D37" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="E37" s="16"/>
+      <c r="F37" s="114"/>
+    </row>
+    <row r="38" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="161"/>
+      <c r="B38" s="163"/>
+      <c r="C38" s="138"/>
+      <c r="D38" s="161"/>
+      <c r="E38" s="162"/>
+      <c r="F38" s="163"/>
+    </row>
+    <row r="39" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="7"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="173"/>
+      <c r="D39" s="152"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+    </row>
+    <row r="40" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="50" t="s">
+        <v>58</v>
+      </c>
+      <c r="B40" s="50" t="s">
+        <v>8</v>
+      </c>
+      <c r="C40" s="185" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" s="175"/>
+      <c r="E40" s="50" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" s="50" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="51" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41" s="51"/>
+      <c r="C41" s="186"/>
+      <c r="D41" s="180"/>
+      <c r="E41" s="51" t="s">
+        <v>59</v>
+      </c>
+      <c r="F41" s="51" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A42" s="139"/>
+      <c r="B42" s="140"/>
+      <c r="C42" s="113"/>
+      <c r="D42" s="114"/>
+      <c r="E42" s="140"/>
+      <c r="F42" s="140"/>
+    </row>
+    <row r="43" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="119"/>
+      <c r="B43" s="120"/>
+      <c r="C43" s="105"/>
+      <c r="D43" s="106"/>
+      <c r="E43" s="187"/>
+      <c r="F43" s="124"/>
+    </row>
+    <row r="44" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="141"/>
+      <c r="B44" s="116"/>
+      <c r="C44" s="105"/>
+      <c r="D44" s="106"/>
+      <c r="E44" s="188"/>
+      <c r="F44" s="116"/>
+    </row>
+    <row r="45" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="119"/>
+      <c r="B45" s="116"/>
+      <c r="C45" s="105"/>
+      <c r="D45" s="106"/>
+      <c r="E45" s="120"/>
+      <c r="F45" s="124"/>
+    </row>
+    <row r="46" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="121"/>
+      <c r="B46" s="116"/>
+      <c r="C46" s="105"/>
+      <c r="D46" s="106"/>
+      <c r="E46" s="106"/>
+      <c r="F46" s="106"/>
+    </row>
+    <row r="47" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="119"/>
+      <c r="B47" s="106"/>
+      <c r="C47" s="105"/>
+      <c r="D47" s="106"/>
+      <c r="E47" s="106"/>
+      <c r="F47" s="106"/>
+    </row>
+    <row r="48" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="119"/>
+      <c r="B48" s="106"/>
+      <c r="C48" s="105"/>
+      <c r="D48" s="106"/>
+      <c r="E48" s="106"/>
+      <c r="F48" s="106"/>
+    </row>
+    <row r="49" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="119"/>
+      <c r="B49" s="106"/>
+      <c r="C49" s="105"/>
+      <c r="D49" s="106"/>
+      <c r="E49" s="106"/>
+      <c r="F49" s="106"/>
+    </row>
+    <row r="50" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="122"/>
+      <c r="B50" s="120"/>
+      <c r="C50" s="105"/>
+      <c r="D50" s="106"/>
+      <c r="E50" s="125"/>
+      <c r="F50" s="116"/>
+    </row>
+    <row r="51" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="122"/>
+      <c r="B51" s="116"/>
+      <c r="C51" s="105"/>
+      <c r="D51" s="106"/>
+      <c r="E51" s="125"/>
+      <c r="F51" s="116"/>
+    </row>
+    <row r="52" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="122"/>
+      <c r="B52" s="116"/>
+      <c r="C52" s="105"/>
+      <c r="D52" s="106"/>
+      <c r="E52" s="125"/>
+      <c r="F52" s="116"/>
+    </row>
+    <row r="53" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="122"/>
+      <c r="B53" s="116"/>
+      <c r="C53" s="105"/>
+      <c r="D53" s="106"/>
+      <c r="E53" s="125"/>
+      <c r="F53" s="116"/>
+    </row>
+    <row r="54" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="122"/>
+      <c r="B54" s="116"/>
+      <c r="C54" s="105"/>
+      <c r="D54" s="106"/>
+      <c r="E54" s="125"/>
+      <c r="F54" s="116"/>
+    </row>
+    <row r="55" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="122"/>
+      <c r="B55" s="120"/>
+      <c r="C55" s="105"/>
+      <c r="D55" s="106"/>
+      <c r="E55" s="125"/>
+      <c r="F55" s="116"/>
+    </row>
+    <row r="56" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="122"/>
+      <c r="B56" s="120"/>
+      <c r="C56" s="105"/>
+      <c r="D56" s="106"/>
+      <c r="E56" s="106"/>
+      <c r="F56" s="125"/>
+    </row>
+    <row r="57" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="122"/>
+      <c r="B57" s="106"/>
+      <c r="C57" s="105"/>
+      <c r="D57" s="106"/>
+      <c r="E57" s="106"/>
+      <c r="F57" s="116"/>
+    </row>
+    <row r="58" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="122"/>
+      <c r="B58" s="106"/>
+      <c r="C58" s="105"/>
+      <c r="D58" s="106"/>
+      <c r="E58" s="120"/>
+      <c r="F58" s="124"/>
+    </row>
+    <row r="59" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="142"/>
+      <c r="B59" s="128"/>
+      <c r="C59" s="126"/>
+      <c r="D59" s="127"/>
+      <c r="E59" s="128"/>
+      <c r="F59" s="124"/>
+    </row>
+    <row r="60" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="143"/>
+      <c r="B60" s="128"/>
+      <c r="C60" s="126"/>
+      <c r="D60" s="127"/>
+      <c r="E60" s="128"/>
+      <c r="F60" s="124"/>
+    </row>
+    <row r="61" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="122"/>
+      <c r="B61" s="120"/>
+      <c r="C61" s="105"/>
+      <c r="D61" s="129"/>
+      <c r="E61" s="120"/>
+      <c r="F61" s="124"/>
+    </row>
+    <row r="62" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="122"/>
+      <c r="B62" s="120"/>
+      <c r="C62" s="105"/>
+      <c r="D62" s="129"/>
+      <c r="E62" s="120"/>
+      <c r="F62" s="124"/>
+    </row>
+    <row r="63" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="122"/>
+      <c r="B63" s="120"/>
+      <c r="C63" s="105"/>
+      <c r="D63" s="129"/>
+      <c r="E63" s="125"/>
+      <c r="F63" s="124"/>
+    </row>
+    <row r="64" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A64" s="123"/>
+      <c r="B64" s="135"/>
+      <c r="C64" s="111"/>
+      <c r="D64" s="130"/>
+      <c r="E64" s="131"/>
+      <c r="F64" s="130"/>
+    </row>
+    <row r="65" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="10"/>
+      <c r="B65" s="83"/>
+      <c r="C65" s="2"/>
+      <c r="D65" s="10"/>
+      <c r="E65" s="84"/>
+      <c r="F65" s="10"/>
+    </row>
+    <row r="66" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A66" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="B66" s="132"/>
+      <c r="C66" s="86" t="s">
+        <v>18</v>
+      </c>
+      <c r="D66" s="87" t="s">
+        <v>19</v>
+      </c>
+      <c r="E66" s="136"/>
+      <c r="F66" s="137"/>
+    </row>
+    <row r="67" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="189"/>
+      <c r="B67" s="190"/>
+      <c r="C67" s="144"/>
+      <c r="D67" s="91"/>
+      <c r="E67" s="11"/>
+      <c r="F67" s="92"/>
+    </row>
+    <row r="68" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="133"/>
+      <c r="B68" s="129"/>
+      <c r="C68" s="94" t="s">
+        <v>20</v>
+      </c>
+      <c r="D68" s="10"/>
+      <c r="E68" s="12"/>
+      <c r="F68" s="74"/>
+    </row>
+    <row r="69" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="134"/>
+      <c r="B69" s="130"/>
+      <c r="C69" s="145"/>
+      <c r="D69" s="10"/>
+      <c r="E69" s="13"/>
+      <c r="F69" s="74"/>
+    </row>
+    <row r="70" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A70" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="B70" s="132"/>
+      <c r="C70" s="86" t="s">
+        <v>43</v>
+      </c>
+      <c r="D70" s="10"/>
+      <c r="E70" s="12"/>
+      <c r="F70" s="74"/>
+    </row>
+    <row r="71" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="191"/>
+      <c r="B71" s="192"/>
+      <c r="C71" s="146"/>
+      <c r="D71" s="10"/>
+      <c r="E71" s="10"/>
+      <c r="F71" s="74"/>
+    </row>
+    <row r="72" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A72" s="18"/>
+      <c r="B72" s="1"/>
+      <c r="C72" s="1"/>
+      <c r="D72" s="193"/>
+      <c r="E72" s="152"/>
+      <c r="F72" s="177"/>
+    </row>
+    <row r="73" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A73" s="98"/>
+      <c r="F73" s="99"/>
+    </row>
+    <row r="74" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A74" s="98"/>
+      <c r="F74" s="99"/>
+    </row>
+    <row r="75" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A75" s="98"/>
+      <c r="D75" s="184" t="s">
+        <v>22</v>
+      </c>
+      <c r="E75" s="152"/>
+      <c r="F75" s="177"/>
+    </row>
+    <row r="76" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="100" t="s">
+        <v>23</v>
+      </c>
+      <c r="B76" s="14"/>
+      <c r="C76" s="14"/>
+      <c r="D76" s="14"/>
+      <c r="E76" s="14"/>
+      <c r="F76" s="101"/>
+    </row>
+  </sheetData>
+  <mergeCells count="40">
+    <mergeCell ref="A67:B67"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="D72:F72"/>
+    <mergeCell ref="D75:F75"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="D38:F38"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D25:F34"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D18:F19"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="D2:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup scale="55" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E734C38C-3C74-4506-B383-F7FA1189C248}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -1924,10 +2562,10 @@
       <c r="A2" s="15"/>
       <c r="B2" s="16"/>
       <c r="C2" s="17"/>
-      <c r="D2" s="188" t="s">
+      <c r="D2" s="150" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="163"/>
+      <c r="E2" s="151"/>
       <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
@@ -1936,8 +2574,8 @@
       <c r="C3" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="148"/>
-      <c r="E3" s="148"/>
+      <c r="D3" s="152"/>
+      <c r="E3" s="152"/>
       <c r="F3" s="20"/>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1946,8 +2584,8 @@
       <c r="C4" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="148"/>
-      <c r="E4" s="148"/>
+      <c r="D4" s="152"/>
+      <c r="E4" s="152"/>
       <c r="F4" s="20"/>
     </row>
     <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1956,8 +2594,8 @@
       <c r="C5" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="148"/>
-      <c r="E5" s="148"/>
+      <c r="D5" s="152"/>
+      <c r="E5" s="152"/>
       <c r="F5" s="20"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1966,20 +2604,20 @@
       <c r="C6" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="189" t="s">
+      <c r="D6" s="153" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="148"/>
+      <c r="E6" s="152"/>
       <c r="F6" s="20"/>
     </row>
     <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="18"/>
       <c r="B7" s="1"/>
       <c r="C7" s="20"/>
-      <c r="D7" s="190" t="s">
-        <v>2</v>
-      </c>
-      <c r="E7" s="148"/>
+      <c r="D7" s="154" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="152"/>
       <c r="F7" s="20"/>
     </row>
     <row r="8" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -2003,24 +2641,24 @@
       <c r="F9" s="114"/>
     </row>
     <row r="10" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="167" t="s">
+      <c r="A10" s="147" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="168"/>
-      <c r="C10" s="169"/>
-      <c r="D10" s="167"/>
-      <c r="E10" s="168"/>
-      <c r="F10" s="169"/>
+      <c r="B10" s="148"/>
+      <c r="C10" s="149"/>
+      <c r="D10" s="147"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="149"/>
     </row>
     <row r="11" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="167" t="s">
+      <c r="A11" s="147" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="168"/>
-      <c r="C11" s="169"/>
-      <c r="D11" s="167"/>
-      <c r="E11" s="168"/>
-      <c r="F11" s="169"/>
+      <c r="B11" s="148"/>
+      <c r="C11" s="149"/>
+      <c r="D11" s="147"/>
+      <c r="E11" s="148"/>
+      <c r="F11" s="149"/>
     </row>
     <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="104"/>
@@ -2056,17 +2694,17 @@
         <v>5</v>
       </c>
       <c r="C15" s="106"/>
-      <c r="D15" s="182"/>
-      <c r="E15" s="183"/>
-      <c r="F15" s="184"/>
+      <c r="D15" s="158"/>
+      <c r="E15" s="159"/>
+      <c r="F15" s="160"/>
     </row>
     <row r="16" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="110"/>
       <c r="B16" s="111"/>
       <c r="C16" s="112"/>
-      <c r="D16" s="173"/>
-      <c r="E16" s="178"/>
-      <c r="F16" s="174"/>
+      <c r="D16" s="161"/>
+      <c r="E16" s="162"/>
+      <c r="F16" s="163"/>
     </row>
     <row r="17" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A17" s="24" t="s">
@@ -2080,34 +2718,34 @@
       <c r="E17" s="113"/>
       <c r="F17" s="114"/>
     </row>
-    <row r="18" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="185"/>
-      <c r="B18" s="186"/>
-      <c r="C18" s="187"/>
-      <c r="D18" s="182"/>
-      <c r="E18" s="183"/>
-      <c r="F18" s="184"/>
-    </row>
-    <row r="19" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="185"/>
-      <c r="B19" s="186"/>
-      <c r="C19" s="187"/>
-      <c r="D19" s="182"/>
-      <c r="E19" s="183"/>
-      <c r="F19" s="184"/>
+    <row r="18" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="164"/>
+      <c r="B18" s="165"/>
+      <c r="C18" s="166"/>
+      <c r="D18" s="170"/>
+      <c r="E18" s="171"/>
+      <c r="F18" s="172"/>
+    </row>
+    <row r="19" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="164"/>
+      <c r="B19" s="165"/>
+      <c r="C19" s="166"/>
+      <c r="D19" s="170"/>
+      <c r="E19" s="171"/>
+      <c r="F19" s="172"/>
     </row>
     <row r="20" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="185"/>
-      <c r="B20" s="186"/>
-      <c r="C20" s="187"/>
-      <c r="D20" s="173"/>
-      <c r="E20" s="178"/>
-      <c r="F20" s="174"/>
+      <c r="A20" s="164"/>
+      <c r="B20" s="165"/>
+      <c r="C20" s="166"/>
+      <c r="D20" s="167"/>
+      <c r="E20" s="168"/>
+      <c r="F20" s="169"/>
     </row>
     <row r="21" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="185"/>
-      <c r="B21" s="186"/>
-      <c r="C21" s="187"/>
+      <c r="A21" s="164"/>
+      <c r="B21" s="165"/>
+      <c r="C21" s="166"/>
       <c r="D21" s="24" t="s">
         <v>51</v>
       </c>
@@ -2115,25 +2753,25 @@
       <c r="F21" s="114"/>
     </row>
     <row r="22" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="167"/>
-      <c r="B22" s="168"/>
-      <c r="C22" s="169"/>
+      <c r="A22" s="170"/>
+      <c r="B22" s="171"/>
+      <c r="C22" s="172"/>
       <c r="D22" s="117"/>
       <c r="E22" s="105"/>
       <c r="F22" s="106"/>
     </row>
     <row r="23" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="167"/>
-      <c r="B23" s="168"/>
-      <c r="C23" s="169"/>
+      <c r="A23" s="170"/>
+      <c r="B23" s="171"/>
+      <c r="C23" s="172"/>
       <c r="D23" s="117"/>
       <c r="E23" s="105"/>
       <c r="F23" s="106"/>
     </row>
     <row r="24" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="179"/>
-      <c r="B24" s="180"/>
-      <c r="C24" s="181"/>
+      <c r="A24" s="155"/>
+      <c r="B24" s="156"/>
+      <c r="C24" s="157"/>
       <c r="D24" s="115"/>
       <c r="E24" s="111"/>
       <c r="F24" s="112"/>
@@ -2144,67 +2782,67 @@
       </c>
       <c r="B25" s="113"/>
       <c r="C25" s="118"/>
-      <c r="D25" s="162" t="s">
+      <c r="D25" s="174" t="s">
         <v>6</v>
       </c>
-      <c r="E25" s="163"/>
-      <c r="F25" s="151"/>
+      <c r="E25" s="151"/>
+      <c r="F25" s="175"/>
     </row>
     <row r="26" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="167"/>
-      <c r="B26" s="168"/>
-      <c r="C26" s="169"/>
-      <c r="D26" s="164"/>
-      <c r="E26" s="148"/>
-      <c r="F26" s="149"/>
+      <c r="A26" s="170"/>
+      <c r="B26" s="171"/>
+      <c r="C26" s="172"/>
+      <c r="D26" s="176"/>
+      <c r="E26" s="152"/>
+      <c r="F26" s="177"/>
     </row>
     <row r="27" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="167"/>
-      <c r="B27" s="168"/>
-      <c r="C27" s="169"/>
-      <c r="D27" s="164"/>
-      <c r="E27" s="148"/>
-      <c r="F27" s="149"/>
+      <c r="A27" s="170"/>
+      <c r="B27" s="171"/>
+      <c r="C27" s="172"/>
+      <c r="D27" s="176"/>
+      <c r="E27" s="152"/>
+      <c r="F27" s="177"/>
     </row>
     <row r="28" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="167"/>
-      <c r="B28" s="168"/>
-      <c r="C28" s="169"/>
-      <c r="D28" s="164"/>
-      <c r="E28" s="148"/>
-      <c r="F28" s="149"/>
+      <c r="A28" s="170"/>
+      <c r="B28" s="171"/>
+      <c r="C28" s="172"/>
+      <c r="D28" s="176"/>
+      <c r="E28" s="152"/>
+      <c r="F28" s="177"/>
     </row>
     <row r="29" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="167"/>
-      <c r="B29" s="168"/>
-      <c r="C29" s="169"/>
-      <c r="D29" s="164"/>
-      <c r="E29" s="148"/>
-      <c r="F29" s="149"/>
+      <c r="A29" s="170"/>
+      <c r="B29" s="171"/>
+      <c r="C29" s="172"/>
+      <c r="D29" s="176"/>
+      <c r="E29" s="152"/>
+      <c r="F29" s="177"/>
     </row>
     <row r="30" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="167"/>
-      <c r="B30" s="168"/>
-      <c r="C30" s="169"/>
-      <c r="D30" s="164"/>
-      <c r="E30" s="148"/>
-      <c r="F30" s="149"/>
+      <c r="A30" s="170"/>
+      <c r="B30" s="171"/>
+      <c r="C30" s="172"/>
+      <c r="D30" s="176"/>
+      <c r="E30" s="152"/>
+      <c r="F30" s="177"/>
     </row>
     <row r="31" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="167"/>
-      <c r="B31" s="168"/>
-      <c r="C31" s="169"/>
-      <c r="D31" s="164"/>
-      <c r="E31" s="148"/>
-      <c r="F31" s="149"/>
+      <c r="A31" s="170"/>
+      <c r="B31" s="171"/>
+      <c r="C31" s="172"/>
+      <c r="D31" s="176"/>
+      <c r="E31" s="152"/>
+      <c r="F31" s="177"/>
     </row>
     <row r="32" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="170"/>
-      <c r="B32" s="171"/>
-      <c r="C32" s="172"/>
-      <c r="D32" s="164"/>
-      <c r="E32" s="148"/>
-      <c r="F32" s="149"/>
+      <c r="A32" s="167"/>
+      <c r="B32" s="168"/>
+      <c r="C32" s="169"/>
+      <c r="D32" s="176"/>
+      <c r="E32" s="152"/>
+      <c r="F32" s="177"/>
     </row>
     <row r="33" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A33" s="24" t="s">
@@ -2214,23 +2852,23 @@
       <c r="C33" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="D33" s="164"/>
-      <c r="E33" s="148"/>
-      <c r="F33" s="149"/>
+      <c r="D33" s="176"/>
+      <c r="E33" s="152"/>
+      <c r="F33" s="177"/>
     </row>
     <row r="34" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="173"/>
-      <c r="B34" s="174"/>
+      <c r="A34" s="161"/>
+      <c r="B34" s="163"/>
       <c r="C34" s="123"/>
-      <c r="D34" s="165"/>
-      <c r="E34" s="166"/>
-      <c r="F34" s="153"/>
+      <c r="D34" s="178"/>
+      <c r="E34" s="179"/>
+      <c r="F34" s="180"/>
     </row>
     <row r="35" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A35" s="175" t="s">
+      <c r="A35" s="181" t="s">
         <v>47</v>
       </c>
-      <c r="B35" s="151"/>
+      <c r="B35" s="175"/>
       <c r="C35" s="46" t="s">
         <v>48</v>
       </c>
@@ -2241,12 +2879,12 @@
       <c r="F35" s="114"/>
     </row>
     <row r="36" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="176"/>
-      <c r="B36" s="177"/>
+      <c r="A36" s="182"/>
+      <c r="B36" s="183"/>
       <c r="C36" s="103"/>
-      <c r="D36" s="173"/>
-      <c r="E36" s="178"/>
-      <c r="F36" s="174"/>
+      <c r="D36" s="161"/>
+      <c r="E36" s="162"/>
+      <c r="F36" s="163"/>
     </row>
     <row r="37" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A37" s="24" t="s">
@@ -2263,18 +2901,18 @@
       <c r="F37" s="114"/>
     </row>
     <row r="38" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="173"/>
-      <c r="B38" s="174"/>
+      <c r="A38" s="161"/>
+      <c r="B38" s="163"/>
       <c r="C38" s="138"/>
-      <c r="D38" s="173"/>
-      <c r="E38" s="178"/>
-      <c r="F38" s="174"/>
+      <c r="D38" s="161"/>
+      <c r="E38" s="162"/>
+      <c r="F38" s="163"/>
     </row>
     <row r="39" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
-      <c r="C39" s="161"/>
-      <c r="D39" s="148"/>
+      <c r="C39" s="173"/>
+      <c r="D39" s="152"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
     </row>
@@ -2285,10 +2923,10 @@
       <c r="B40" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="150" t="s">
+      <c r="C40" s="185" t="s">
         <v>9</v>
       </c>
-      <c r="D40" s="151"/>
+      <c r="D40" s="175"/>
       <c r="E40" s="50" t="s">
         <v>10</v>
       </c>
@@ -2301,8 +2939,8 @@
         <v>7</v>
       </c>
       <c r="B41" s="51"/>
-      <c r="C41" s="152"/>
-      <c r="D41" s="153"/>
+      <c r="C41" s="186"/>
+      <c r="D41" s="180"/>
       <c r="E41" s="51" t="s">
         <v>59</v>
       </c>
@@ -2323,7 +2961,7 @@
       <c r="B43" s="120"/>
       <c r="C43" s="105"/>
       <c r="D43" s="106"/>
-      <c r="E43" s="154"/>
+      <c r="E43" s="187"/>
       <c r="F43" s="124"/>
     </row>
     <row r="44" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2331,7 +2969,7 @@
       <c r="B44" s="116"/>
       <c r="C44" s="105"/>
       <c r="D44" s="106"/>
-      <c r="E44" s="155"/>
+      <c r="E44" s="188"/>
       <c r="F44" s="116"/>
     </row>
     <row r="45" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2517,8 +3155,8 @@
       <c r="F66" s="137"/>
     </row>
     <row r="67" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="156"/>
-      <c r="B67" s="157"/>
+      <c r="A67" s="189"/>
+      <c r="B67" s="190"/>
       <c r="C67" s="144"/>
       <c r="D67" s="91"/>
       <c r="E67" s="11"/>
@@ -2555,8 +3193,8 @@
       <c r="F70" s="74"/>
     </row>
     <row r="71" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="158"/>
-      <c r="B71" s="159"/>
+      <c r="A71" s="191"/>
+      <c r="B71" s="192"/>
       <c r="C71" s="146"/>
       <c r="D71" s="10"/>
       <c r="E71" s="10"/>
@@ -2566,9 +3204,9 @@
       <c r="A72" s="18"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
-      <c r="D72" s="160"/>
-      <c r="E72" s="148"/>
-      <c r="F72" s="149"/>
+      <c r="D72" s="193"/>
+      <c r="E72" s="152"/>
+      <c r="F72" s="177"/>
     </row>
     <row r="73" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="98"/>
@@ -2580,11 +3218,11 @@
     </row>
     <row r="75" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A75" s="98"/>
-      <c r="D75" s="147" t="s">
+      <c r="D75" s="184" t="s">
         <v>22</v>
       </c>
-      <c r="E75" s="148"/>
-      <c r="F75" s="149"/>
+      <c r="E75" s="152"/>
+      <c r="F75" s="177"/>
     </row>
     <row r="76" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="100" t="s">
@@ -2597,26 +3235,14 @@
       <c r="F76" s="101"/>
     </row>
   </sheetData>
-  <mergeCells count="41">
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D2:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A23:C23"/>
+  <mergeCells count="40">
+    <mergeCell ref="D75:F75"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="A67:B67"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="D72:F72"/>
     <mergeCell ref="C39:D39"/>
     <mergeCell ref="D25:F34"/>
     <mergeCell ref="A26:C26"/>
@@ -2632,760 +3258,24 @@
     <mergeCell ref="D36:F36"/>
     <mergeCell ref="A38:B38"/>
     <mergeCell ref="D38:F38"/>
-    <mergeCell ref="D75:F75"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="A67:B67"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="D72:F72"/>
-  </mergeCells>
-  <printOptions horizontalCentered="1" verticalCentered="1"/>
-  <pageMargins left="0.25" right="0.25" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup scale="55" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:F76"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="23.75" customWidth="1"/>
-    <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="44.25" customWidth="1"/>
-    <col min="4" max="4" width="28.75" customWidth="1"/>
-    <col min="5" max="6" width="27.25" customWidth="1"/>
-    <col min="7" max="25" width="10.625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="14"/>
-      <c r="F1" s="14"/>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="15"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="188" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="163"/>
-      <c r="F2" s="17"/>
-    </row>
-    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="18"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" s="148"/>
-      <c r="E3" s="148"/>
-      <c r="F3" s="20"/>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="18"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" s="148"/>
-      <c r="E4" s="148"/>
-      <c r="F4" s="20"/>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="18"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="148"/>
-      <c r="E5" s="148"/>
-      <c r="F5" s="20"/>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="18"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="189" t="s">
-        <v>1</v>
-      </c>
-      <c r="E6" s="148"/>
-      <c r="F6" s="20"/>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="18"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="190" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="148"/>
-      <c r="F7" s="20"/>
-    </row>
-    <row r="8" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="21"/>
-      <c r="B8" s="22"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="23"/>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="25"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="16"/>
-      <c r="F9" s="17"/>
-    </row>
-    <row r="10" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="211" t="s">
-        <v>61</v>
-      </c>
-      <c r="B10" s="212"/>
-      <c r="C10" s="213"/>
-      <c r="D10" s="221"/>
-      <c r="E10" s="222"/>
-      <c r="F10" s="223"/>
-    </row>
-    <row r="11" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="211" t="s">
-        <v>62</v>
-      </c>
-      <c r="B11" s="212"/>
-      <c r="C11" s="213"/>
-      <c r="D11" s="221"/>
-      <c r="E11" s="222"/>
-      <c r="F11" s="223"/>
-    </row>
-    <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="30" t="s">
-        <v>3</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="20"/>
-    </row>
-    <row r="13" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="31"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="23"/>
-    </row>
-    <row r="14" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="28"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="E14" s="16"/>
-      <c r="F14" s="17"/>
-    </row>
-    <row r="15" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="32"/>
-      <c r="B15" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="224"/>
-      <c r="E15" s="160"/>
-      <c r="F15" s="225"/>
-    </row>
-    <row r="16" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="33"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="204"/>
-      <c r="E16" s="205"/>
-      <c r="F16" s="206"/>
-    </row>
-    <row r="17" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="B17" s="25"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="34" t="s">
-        <v>52</v>
-      </c>
-      <c r="E17" s="16"/>
-      <c r="F17" s="17"/>
-    </row>
-    <row r="18" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="195"/>
-      <c r="B18" s="196"/>
-      <c r="C18" s="197"/>
-      <c r="D18" s="226"/>
-      <c r="E18" s="227"/>
-      <c r="F18" s="228"/>
-    </row>
-    <row r="19" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="195"/>
-      <c r="B19" s="196"/>
-      <c r="C19" s="197"/>
-      <c r="D19" s="226"/>
-      <c r="E19" s="227"/>
-      <c r="F19" s="228"/>
-    </row>
-    <row r="20" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="195"/>
-      <c r="B20" s="196"/>
-      <c r="C20" s="197"/>
-      <c r="D20" s="229"/>
-      <c r="E20" s="230"/>
-      <c r="F20" s="231"/>
-    </row>
-    <row r="21" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="195"/>
-      <c r="B21" s="196"/>
-      <c r="C21" s="197"/>
-      <c r="D21" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="E21" s="16"/>
-      <c r="F21" s="17"/>
-    </row>
-    <row r="22" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="198"/>
-      <c r="B22" s="199"/>
-      <c r="C22" s="200"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="20"/>
-    </row>
-    <row r="23" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="198"/>
-      <c r="B23" s="199"/>
-      <c r="C23" s="200"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="20"/>
-    </row>
-    <row r="24" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="207"/>
-      <c r="B24" s="208"/>
-      <c r="C24" s="209"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="23"/>
-    </row>
-    <row r="25" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="B25" s="41"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="162" t="s">
-        <v>6</v>
-      </c>
-      <c r="E25" s="163"/>
-      <c r="F25" s="151"/>
-    </row>
-    <row r="26" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="214"/>
-      <c r="B26" s="215"/>
-      <c r="C26" s="216"/>
-      <c r="D26" s="164"/>
-      <c r="E26" s="148"/>
-      <c r="F26" s="149"/>
-    </row>
-    <row r="27" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="198"/>
-      <c r="B27" s="199"/>
-      <c r="C27" s="200"/>
-      <c r="D27" s="164"/>
-      <c r="E27" s="148"/>
-      <c r="F27" s="149"/>
-    </row>
-    <row r="28" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="198"/>
-      <c r="B28" s="199"/>
-      <c r="C28" s="200"/>
-      <c r="D28" s="164"/>
-      <c r="E28" s="148"/>
-      <c r="F28" s="149"/>
-    </row>
-    <row r="29" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="198"/>
-      <c r="B29" s="199"/>
-      <c r="C29" s="200"/>
-      <c r="D29" s="164"/>
-      <c r="E29" s="148"/>
-      <c r="F29" s="149"/>
-    </row>
-    <row r="30" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="198"/>
-      <c r="B30" s="199"/>
-      <c r="C30" s="200"/>
-      <c r="D30" s="164"/>
-      <c r="E30" s="148"/>
-      <c r="F30" s="149"/>
-    </row>
-    <row r="31" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="198"/>
-      <c r="B31" s="199"/>
-      <c r="C31" s="200"/>
-      <c r="D31" s="164"/>
-      <c r="E31" s="148"/>
-      <c r="F31" s="149"/>
-    </row>
-    <row r="32" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="217"/>
-      <c r="B32" s="218"/>
-      <c r="C32" s="219"/>
-      <c r="D32" s="164"/>
-      <c r="E32" s="148"/>
-      <c r="F32" s="149"/>
-    </row>
-    <row r="33" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="B33" s="16"/>
-      <c r="C33" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="D33" s="164"/>
-      <c r="E33" s="148"/>
-      <c r="F33" s="149"/>
-    </row>
-    <row r="34" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="201"/>
-      <c r="B34" s="202"/>
-      <c r="C34" s="47"/>
-      <c r="D34" s="165"/>
-      <c r="E34" s="166"/>
-      <c r="F34" s="153"/>
-    </row>
-    <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="175" t="s">
-        <v>47</v>
-      </c>
-      <c r="B35" s="151"/>
-      <c r="C35" s="46" t="s">
-        <v>48</v>
-      </c>
-      <c r="D35" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="E35" s="16"/>
-      <c r="F35" s="17"/>
-    </row>
-    <row r="36" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="210"/>
-      <c r="B36" s="153"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="204"/>
-      <c r="E36" s="205"/>
-      <c r="F36" s="206"/>
-    </row>
-    <row r="37" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A37" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="B37" s="48"/>
-      <c r="C37" s="46" t="s">
-        <v>45</v>
-      </c>
-      <c r="D37" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E37" s="16"/>
-      <c r="F37" s="17"/>
-    </row>
-    <row r="38" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="201"/>
-      <c r="B38" s="202"/>
-      <c r="C38" s="49"/>
-      <c r="D38" s="201"/>
-      <c r="E38" s="203"/>
-      <c r="F38" s="202"/>
-    </row>
-    <row r="39" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="7"/>
-      <c r="B39" s="7"/>
-      <c r="C39" s="161"/>
-      <c r="D39" s="148"/>
-      <c r="E39" s="7"/>
-      <c r="F39" s="7"/>
-    </row>
-    <row r="40" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="50" t="s">
-        <v>58</v>
-      </c>
-      <c r="B40" s="50" t="s">
-        <v>8</v>
-      </c>
-      <c r="C40" s="150" t="s">
-        <v>9</v>
-      </c>
-      <c r="D40" s="151"/>
-      <c r="E40" s="50" t="s">
-        <v>10</v>
-      </c>
-      <c r="F40" s="50" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="51" t="s">
-        <v>7</v>
-      </c>
-      <c r="B41" s="51"/>
-      <c r="C41" s="152"/>
-      <c r="D41" s="153"/>
-      <c r="E41" s="51" t="s">
-        <v>59</v>
-      </c>
-      <c r="F41" s="51" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="52"/>
-      <c r="B42" s="53"/>
-      <c r="C42" s="54"/>
-      <c r="D42" s="17"/>
-      <c r="E42" s="53"/>
-      <c r="F42" s="53"/>
-    </row>
-    <row r="43" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="55"/>
-      <c r="B43" s="56"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="57"/>
-      <c r="E43" s="220"/>
-      <c r="F43" s="58"/>
-    </row>
-    <row r="44" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="59"/>
-      <c r="B44" s="60"/>
-      <c r="C44" s="1"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="149"/>
-      <c r="F44" s="60"/>
-    </row>
-    <row r="45" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="55"/>
-      <c r="B45" s="61"/>
-      <c r="C45" s="1"/>
-      <c r="D45" s="20"/>
-      <c r="E45" s="62"/>
-      <c r="F45" s="63"/>
-    </row>
-    <row r="46" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="64"/>
-      <c r="B46" s="60"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="20"/>
-      <c r="E46" s="20"/>
-      <c r="F46" s="20"/>
-    </row>
-    <row r="47" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="55"/>
-      <c r="B47" s="20"/>
-      <c r="C47" s="1"/>
-      <c r="D47" s="20"/>
-      <c r="E47" s="20"/>
-      <c r="F47" s="20"/>
-    </row>
-    <row r="48" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="55"/>
-      <c r="B48" s="20"/>
-      <c r="C48" s="1"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="20"/>
-      <c r="F48" s="20"/>
-    </row>
-    <row r="49" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="55"/>
-      <c r="B49" s="20"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="20"/>
-      <c r="E49" s="20"/>
-      <c r="F49" s="20"/>
-    </row>
-    <row r="50" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="65"/>
-      <c r="B50" s="56"/>
-      <c r="C50" s="1"/>
-      <c r="D50" s="20"/>
-      <c r="E50" s="66"/>
-      <c r="F50" s="60"/>
-    </row>
-    <row r="51" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="65"/>
-      <c r="B51" s="60"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="20"/>
-      <c r="E51" s="66"/>
-      <c r="F51" s="60"/>
-    </row>
-    <row r="52" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="65"/>
-      <c r="B52" s="60"/>
-      <c r="C52" s="1"/>
-      <c r="D52" s="20"/>
-      <c r="E52" s="66"/>
-      <c r="F52" s="60"/>
-    </row>
-    <row r="53" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="65"/>
-      <c r="B53" s="60"/>
-      <c r="C53" s="1"/>
-      <c r="D53" s="20"/>
-      <c r="E53" s="66"/>
-      <c r="F53" s="60"/>
-    </row>
-    <row r="54" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="65"/>
-      <c r="B54" s="60"/>
-      <c r="C54" s="1"/>
-      <c r="D54" s="20"/>
-      <c r="E54" s="66"/>
-      <c r="F54" s="60"/>
-    </row>
-    <row r="55" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="65"/>
-      <c r="B55" s="56"/>
-      <c r="C55" s="1"/>
-      <c r="D55" s="20"/>
-      <c r="E55" s="66"/>
-      <c r="F55" s="60"/>
-    </row>
-    <row r="56" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="65"/>
-      <c r="B56" s="56"/>
-      <c r="C56" s="1"/>
-      <c r="D56" s="20"/>
-      <c r="E56" s="20"/>
-      <c r="F56" s="66"/>
-    </row>
-    <row r="57" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="65"/>
-      <c r="B57" s="20"/>
-      <c r="C57" s="1"/>
-      <c r="D57" s="20"/>
-      <c r="E57" s="20"/>
-      <c r="F57" s="60"/>
-    </row>
-    <row r="58" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="67"/>
-      <c r="B58" s="20"/>
-      <c r="C58" s="6"/>
-      <c r="D58" s="68"/>
-      <c r="E58" s="62"/>
-      <c r="F58" s="63"/>
-    </row>
-    <row r="59" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="69"/>
-      <c r="B59" s="70"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="71"/>
-      <c r="E59" s="70"/>
-      <c r="F59" s="63"/>
-    </row>
-    <row r="60" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="72"/>
-      <c r="B60" s="70"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="71"/>
-      <c r="E60" s="73"/>
-      <c r="F60" s="63"/>
-    </row>
-    <row r="61" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="67"/>
-      <c r="B61" s="62"/>
-      <c r="C61" s="1"/>
-      <c r="D61" s="74"/>
-      <c r="E61" s="62"/>
-      <c r="F61" s="63"/>
-    </row>
-    <row r="62" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="75"/>
-      <c r="B62" s="62"/>
-      <c r="C62" s="1"/>
-      <c r="D62" s="74"/>
-      <c r="E62" s="62"/>
-      <c r="F62" s="63"/>
-    </row>
-    <row r="63" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="75"/>
-      <c r="B63" s="76"/>
-      <c r="C63" s="2"/>
-      <c r="D63" s="74"/>
-      <c r="E63" s="77"/>
-      <c r="F63" s="63"/>
-    </row>
-    <row r="64" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="78"/>
-      <c r="B64" s="79"/>
-      <c r="C64" s="80"/>
-      <c r="D64" s="81"/>
-      <c r="E64" s="82"/>
-      <c r="F64" s="81"/>
-    </row>
-    <row r="65" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="10"/>
-      <c r="B65" s="83"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="10"/>
-      <c r="E65" s="84"/>
-      <c r="F65" s="10"/>
-    </row>
-    <row r="66" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A66" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="B66" s="85"/>
-      <c r="C66" s="86" t="s">
-        <v>18</v>
-      </c>
-      <c r="D66" s="87" t="s">
-        <v>19</v>
-      </c>
-      <c r="E66" s="88"/>
-      <c r="F66" s="48"/>
-    </row>
-    <row r="67" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="191"/>
-      <c r="B67" s="192"/>
-      <c r="C67" s="90"/>
-      <c r="D67" s="91"/>
-      <c r="E67" s="11"/>
-      <c r="F67" s="92"/>
-    </row>
-    <row r="68" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="93"/>
-      <c r="B68" s="74"/>
-      <c r="C68" s="94" t="s">
-        <v>20</v>
-      </c>
-      <c r="D68" s="10"/>
-      <c r="E68" s="12"/>
-      <c r="F68" s="74"/>
-    </row>
-    <row r="69" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="95"/>
-      <c r="B69" s="81"/>
-      <c r="C69" s="96"/>
-      <c r="D69" s="10"/>
-      <c r="E69" s="13"/>
-      <c r="F69" s="74"/>
-    </row>
-    <row r="70" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A70" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="B70" s="85"/>
-      <c r="C70" s="86" t="s">
-        <v>43</v>
-      </c>
-      <c r="D70" s="10"/>
-      <c r="E70" s="12"/>
-      <c r="F70" s="74"/>
-    </row>
-    <row r="71" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="193"/>
-      <c r="B71" s="194"/>
-      <c r="C71" s="97"/>
-      <c r="D71" s="10"/>
-      <c r="E71" s="10"/>
-      <c r="F71" s="74"/>
-    </row>
-    <row r="72" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A72" s="18"/>
-      <c r="B72" s="1"/>
-      <c r="C72" s="1"/>
-      <c r="D72" s="160"/>
-      <c r="E72" s="148"/>
-      <c r="F72" s="149"/>
-    </row>
-    <row r="73" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A73" s="98"/>
-      <c r="F73" s="99"/>
-    </row>
-    <row r="74" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A74" s="98"/>
-      <c r="F74" s="99"/>
-    </row>
-    <row r="75" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A75" s="98"/>
-      <c r="D75" s="147" t="s">
-        <v>22</v>
-      </c>
-      <c r="E75" s="148"/>
-      <c r="F75" s="149"/>
-    </row>
-    <row r="76" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="100" t="s">
-        <v>23</v>
-      </c>
-      <c r="B76" s="14"/>
-      <c r="C76" s="14"/>
-      <c r="D76" s="14"/>
-      <c r="E76" s="14"/>
-      <c r="F76" s="101"/>
-    </row>
-  </sheetData>
-  <mergeCells count="41">
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="D72:F72"/>
-    <mergeCell ref="D75:F75"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="D18:F19"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
     <mergeCell ref="D2:E5"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D25:F34"/>
+    <mergeCell ref="A10:C10"/>
     <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A67:B67"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="D38:F38"/>
-    <mergeCell ref="D36:F36"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A36:B36"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0" bottom="0" header="0" footer="0"/>
@@ -3415,10 +3305,10 @@
       <c r="A2" s="15"/>
       <c r="B2" s="16"/>
       <c r="C2" s="17"/>
-      <c r="D2" s="188" t="s">
+      <c r="D2" s="150" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="163"/>
+      <c r="E2" s="151"/>
       <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
@@ -3427,8 +3317,8 @@
       <c r="C3" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="148"/>
-      <c r="E3" s="148"/>
+      <c r="D3" s="152"/>
+      <c r="E3" s="152"/>
       <c r="F3" s="20"/>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3437,8 +3327,8 @@
       <c r="C4" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="148"/>
-      <c r="E4" s="148"/>
+      <c r="D4" s="152"/>
+      <c r="E4" s="152"/>
       <c r="F4" s="20"/>
     </row>
     <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3447,8 +3337,8 @@
       <c r="C5" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="148"/>
-      <c r="E5" s="148"/>
+      <c r="D5" s="152"/>
+      <c r="E5" s="152"/>
       <c r="F5" s="20"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3457,20 +3347,20 @@
       <c r="C6" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="189" t="s">
+      <c r="D6" s="153" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="148"/>
+      <c r="E6" s="152"/>
       <c r="F6" s="20"/>
     </row>
     <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="18"/>
       <c r="B7" s="1"/>
       <c r="C7" s="20"/>
-      <c r="D7" s="190" t="s">
+      <c r="D7" s="154" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="148"/>
+      <c r="E7" s="152"/>
       <c r="F7" s="20"/>
     </row>
     <row r="8" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3631,67 +3521,67 @@
       </c>
       <c r="B25" s="41"/>
       <c r="C25" s="26"/>
-      <c r="D25" s="162" t="s">
+      <c r="D25" s="174" t="s">
         <v>6</v>
       </c>
-      <c r="E25" s="163"/>
-      <c r="F25" s="151"/>
+      <c r="E25" s="151"/>
+      <c r="F25" s="175"/>
     </row>
     <row r="26" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="42"/>
       <c r="B26" s="7"/>
       <c r="C26" s="43"/>
-      <c r="D26" s="164"/>
-      <c r="E26" s="148"/>
-      <c r="F26" s="149"/>
+      <c r="D26" s="176"/>
+      <c r="E26" s="152"/>
+      <c r="F26" s="177"/>
     </row>
     <row r="27" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="38"/>
       <c r="B27" s="6"/>
       <c r="C27" s="20"/>
-      <c r="D27" s="164"/>
-      <c r="E27" s="148"/>
-      <c r="F27" s="149"/>
+      <c r="D27" s="176"/>
+      <c r="E27" s="152"/>
+      <c r="F27" s="177"/>
     </row>
     <row r="28" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="38"/>
       <c r="B28" s="6"/>
       <c r="C28" s="20"/>
-      <c r="D28" s="164"/>
-      <c r="E28" s="148"/>
-      <c r="F28" s="149"/>
+      <c r="D28" s="176"/>
+      <c r="E28" s="152"/>
+      <c r="F28" s="177"/>
     </row>
     <row r="29" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="38"/>
       <c r="B29" s="6"/>
       <c r="C29" s="20"/>
-      <c r="D29" s="164"/>
-      <c r="E29" s="148"/>
-      <c r="F29" s="149"/>
+      <c r="D29" s="176"/>
+      <c r="E29" s="152"/>
+      <c r="F29" s="177"/>
     </row>
     <row r="30" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="38"/>
       <c r="B30" s="6"/>
       <c r="C30" s="20"/>
-      <c r="D30" s="164"/>
-      <c r="E30" s="148"/>
-      <c r="F30" s="149"/>
+      <c r="D30" s="176"/>
+      <c r="E30" s="152"/>
+      <c r="F30" s="177"/>
     </row>
     <row r="31" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="38"/>
       <c r="B31" s="6"/>
       <c r="C31" s="20"/>
-      <c r="D31" s="164"/>
-      <c r="E31" s="148"/>
-      <c r="F31" s="149"/>
+      <c r="D31" s="176"/>
+      <c r="E31" s="152"/>
+      <c r="F31" s="177"/>
     </row>
     <row r="32" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="44"/>
       <c r="B32" s="22"/>
       <c r="C32" s="45"/>
-      <c r="D32" s="164"/>
-      <c r="E32" s="148"/>
-      <c r="F32" s="149"/>
+      <c r="D32" s="176"/>
+      <c r="E32" s="152"/>
+      <c r="F32" s="177"/>
     </row>
     <row r="33" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="24" t="s">
@@ -3701,23 +3591,23 @@
       <c r="C33" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="D33" s="164"/>
-      <c r="E33" s="148"/>
-      <c r="F33" s="149"/>
+      <c r="D33" s="176"/>
+      <c r="E33" s="152"/>
+      <c r="F33" s="177"/>
     </row>
     <row r="34" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="33"/>
       <c r="B34" s="22"/>
       <c r="C34" s="47"/>
-      <c r="D34" s="165"/>
-      <c r="E34" s="166"/>
-      <c r="F34" s="153"/>
+      <c r="D34" s="178"/>
+      <c r="E34" s="179"/>
+      <c r="F34" s="180"/>
     </row>
     <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="175" t="s">
+      <c r="A35" s="181" t="s">
         <v>47</v>
       </c>
-      <c r="B35" s="151"/>
+      <c r="B35" s="175"/>
       <c r="C35" s="46" t="s">
         <v>48</v>
       </c>
@@ -3728,8 +3618,8 @@
       <c r="F35" s="17"/>
     </row>
     <row r="36" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="210"/>
-      <c r="B36" s="153"/>
+      <c r="A36" s="195"/>
+      <c r="B36" s="180"/>
       <c r="C36" s="47"/>
       <c r="D36" s="21"/>
       <c r="E36" s="22"/>
@@ -3760,8 +3650,8 @@
     <row r="39" spans="1:6" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
-      <c r="C39" s="161"/>
-      <c r="D39" s="148"/>
+      <c r="C39" s="173"/>
+      <c r="D39" s="152"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
     </row>
@@ -3772,10 +3662,10 @@
       <c r="B40" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="150" t="s">
+      <c r="C40" s="185" t="s">
         <v>9</v>
       </c>
-      <c r="D40" s="151"/>
+      <c r="D40" s="175"/>
       <c r="E40" s="50" t="s">
         <v>10</v>
       </c>
@@ -3788,8 +3678,8 @@
         <v>7</v>
       </c>
       <c r="B41" s="51"/>
-      <c r="C41" s="152"/>
-      <c r="D41" s="153"/>
+      <c r="C41" s="186"/>
+      <c r="D41" s="180"/>
       <c r="E41" s="51" t="s">
         <v>59</v>
       </c>
@@ -3810,7 +3700,7 @@
       <c r="B43" s="56"/>
       <c r="C43" s="1"/>
       <c r="D43" s="57"/>
-      <c r="E43" s="220"/>
+      <c r="E43" s="194"/>
       <c r="F43" s="58"/>
     </row>
     <row r="44" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3818,7 +3708,7 @@
       <c r="B44" s="60"/>
       <c r="C44" s="1"/>
       <c r="D44" s="20"/>
-      <c r="E44" s="149"/>
+      <c r="E44" s="177"/>
       <c r="F44" s="60"/>
     </row>
     <row r="45" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4053,9 +3943,9 @@
       <c r="A72" s="18"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
-      <c r="D72" s="160"/>
-      <c r="E72" s="148"/>
-      <c r="F72" s="149"/>
+      <c r="D72" s="193"/>
+      <c r="E72" s="152"/>
+      <c r="F72" s="177"/>
     </row>
     <row r="73" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="98"/>
@@ -4067,11 +3957,11 @@
     </row>
     <row r="75" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A75" s="98"/>
-      <c r="D75" s="147" t="s">
+      <c r="D75" s="184" t="s">
         <v>22</v>
       </c>
-      <c r="E75" s="148"/>
-      <c r="F75" s="149"/>
+      <c r="E75" s="152"/>
+      <c r="F75" s="177"/>
     </row>
     <row r="76" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="100" t="s">
@@ -4131,10 +4021,10 @@
       <c r="B7" s="15"/>
       <c r="C7" s="16"/>
       <c r="D7" s="17"/>
-      <c r="E7" s="188" t="s">
+      <c r="E7" s="150" t="s">
         <v>0</v>
       </c>
-      <c r="F7" s="163"/>
+      <c r="F7" s="151"/>
       <c r="G7" s="17"/>
     </row>
     <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
@@ -4144,8 +4034,8 @@
       <c r="D8" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="148"/>
-      <c r="F8" s="148"/>
+      <c r="E8" s="152"/>
+      <c r="F8" s="152"/>
       <c r="G8" s="20"/>
     </row>
     <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4155,8 +4045,8 @@
       <c r="D9" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="148"/>
-      <c r="F9" s="148"/>
+      <c r="E9" s="152"/>
+      <c r="F9" s="152"/>
       <c r="G9" s="20"/>
     </row>
     <row r="10" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4166,8 +4056,8 @@
       <c r="D10" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="148"/>
-      <c r="F10" s="148"/>
+      <c r="E10" s="152"/>
+      <c r="F10" s="152"/>
       <c r="G10" s="20"/>
     </row>
     <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4177,10 +4067,10 @@
       <c r="D11" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="189" t="s">
+      <c r="E11" s="153" t="s">
         <v>1</v>
       </c>
-      <c r="F11" s="148"/>
+      <c r="F11" s="152"/>
       <c r="G11" s="20"/>
     </row>
     <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
@@ -4188,10 +4078,10 @@
       <c r="B12" s="18"/>
       <c r="C12" s="1"/>
       <c r="D12" s="20"/>
-      <c r="E12" s="190" t="s">
+      <c r="E12" s="154" t="s">
         <v>42</v>
       </c>
-      <c r="F12" s="148"/>
+      <c r="F12" s="152"/>
       <c r="G12" s="20"/>
     </row>
     <row r="13" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -4370,74 +4260,74 @@
       </c>
       <c r="C30" s="41"/>
       <c r="D30" s="26"/>
-      <c r="E30" s="162" t="s">
+      <c r="E30" s="174" t="s">
         <v>6</v>
       </c>
-      <c r="F30" s="163"/>
-      <c r="G30" s="151"/>
+      <c r="F30" s="151"/>
+      <c r="G30" s="175"/>
     </row>
     <row r="31" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="42"/>
       <c r="C31" s="7"/>
       <c r="D31" s="43"/>
-      <c r="E31" s="164"/>
-      <c r="F31" s="148"/>
-      <c r="G31" s="149"/>
+      <c r="E31" s="176"/>
+      <c r="F31" s="152"/>
+      <c r="G31" s="177"/>
     </row>
     <row r="32" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="38"/>
       <c r="C32" s="6"/>
       <c r="D32" s="20"/>
-      <c r="E32" s="164"/>
-      <c r="F32" s="148"/>
-      <c r="G32" s="149"/>
+      <c r="E32" s="176"/>
+      <c r="F32" s="152"/>
+      <c r="G32" s="177"/>
     </row>
     <row r="33" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="38"/>
       <c r="C33" s="6"/>
       <c r="D33" s="20"/>
-      <c r="E33" s="164"/>
-      <c r="F33" s="148"/>
-      <c r="G33" s="149"/>
+      <c r="E33" s="176"/>
+      <c r="F33" s="152"/>
+      <c r="G33" s="177"/>
     </row>
     <row r="34" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="38"/>
       <c r="C34" s="6"/>
       <c r="D34" s="20"/>
-      <c r="E34" s="164"/>
-      <c r="F34" s="148"/>
-      <c r="G34" s="149"/>
+      <c r="E34" s="176"/>
+      <c r="F34" s="152"/>
+      <c r="G34" s="177"/>
     </row>
     <row r="35" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="38"/>
       <c r="C35" s="6"/>
       <c r="D35" s="20"/>
-      <c r="E35" s="164"/>
-      <c r="F35" s="148"/>
-      <c r="G35" s="149"/>
+      <c r="E35" s="176"/>
+      <c r="F35" s="152"/>
+      <c r="G35" s="177"/>
     </row>
     <row r="36" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="38"/>
       <c r="C36" s="6"/>
       <c r="D36" s="20"/>
-      <c r="E36" s="164"/>
-      <c r="F36" s="148"/>
-      <c r="G36" s="149"/>
+      <c r="E36" s="176"/>
+      <c r="F36" s="152"/>
+      <c r="G36" s="177"/>
     </row>
     <row r="37" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="44"/>
       <c r="C37" s="22"/>
       <c r="D37" s="45"/>
-      <c r="E37" s="164"/>
-      <c r="F37" s="148"/>
-      <c r="G37" s="149"/>
+      <c r="E37" s="176"/>
+      <c r="F37" s="152"/>
+      <c r="G37" s="177"/>
     </row>
     <row r="38" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
@@ -4446,25 +4336,25 @@
       </c>
       <c r="C38" s="16"/>
       <c r="D38" s="17"/>
-      <c r="E38" s="164"/>
-      <c r="F38" s="148"/>
-      <c r="G38" s="149"/>
+      <c r="E38" s="176"/>
+      <c r="F38" s="152"/>
+      <c r="G38" s="177"/>
     </row>
     <row r="39" spans="1:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="33"/>
       <c r="C39" s="22"/>
       <c r="D39" s="40"/>
-      <c r="E39" s="165"/>
-      <c r="F39" s="166"/>
-      <c r="G39" s="153"/>
+      <c r="E39" s="178"/>
+      <c r="F39" s="179"/>
+      <c r="G39" s="180"/>
     </row>
     <row r="40" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="175" t="s">
+      <c r="B40" s="181" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="151"/>
+      <c r="C40" s="175"/>
       <c r="D40" s="46" t="s">
         <v>36</v>
       </c>
@@ -4476,8 +4366,8 @@
     </row>
     <row r="41" spans="1:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
-      <c r="B41" s="210"/>
-      <c r="C41" s="153"/>
+      <c r="B41" s="195"/>
+      <c r="C41" s="180"/>
       <c r="D41" s="47"/>
       <c r="E41" s="21"/>
       <c r="F41" s="22"/>
@@ -4511,8 +4401,8 @@
       <c r="A44" s="1"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
-      <c r="D44" s="161"/>
-      <c r="E44" s="148"/>
+      <c r="D44" s="173"/>
+      <c r="E44" s="152"/>
       <c r="F44" s="7"/>
       <c r="G44" s="7"/>
     </row>
@@ -4524,10 +4414,10 @@
       <c r="C45" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="D45" s="150" t="s">
+      <c r="D45" s="185" t="s">
         <v>9</v>
       </c>
-      <c r="E45" s="151"/>
+      <c r="E45" s="175"/>
       <c r="F45" s="50" t="s">
         <v>10</v>
       </c>
@@ -4543,10 +4433,10 @@
       <c r="C46" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="D46" s="152" t="s">
+      <c r="D46" s="186" t="s">
         <v>14</v>
       </c>
-      <c r="E46" s="153"/>
+      <c r="E46" s="180"/>
       <c r="F46" s="51" t="s">
         <v>15</v>
       </c>
@@ -4569,7 +4459,7 @@
       <c r="C48" s="56"/>
       <c r="D48" s="1"/>
       <c r="E48" s="57"/>
-      <c r="F48" s="220"/>
+      <c r="F48" s="194"/>
       <c r="G48" s="58"/>
     </row>
     <row r="49" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4578,7 +4468,7 @@
       <c r="C49" s="60"/>
       <c r="D49" s="1"/>
       <c r="E49" s="20"/>
-      <c r="F49" s="149"/>
+      <c r="F49" s="177"/>
       <c r="G49" s="60"/>
     </row>
     <row r="50" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4841,9 +4731,9 @@
       <c r="B77" s="18"/>
       <c r="C77" s="1"/>
       <c r="D77" s="1"/>
-      <c r="E77" s="160"/>
-      <c r="F77" s="148"/>
-      <c r="G77" s="149"/>
+      <c r="E77" s="193"/>
+      <c r="F77" s="152"/>
+      <c r="G77" s="177"/>
     </row>
     <row r="78" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B78" s="98"/>
@@ -4855,11 +4745,11 @@
     </row>
     <row r="80" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B80" s="98"/>
-      <c r="E80" s="147" t="s">
+      <c r="E80" s="184" t="s">
         <v>22</v>
       </c>
-      <c r="F80" s="148"/>
-      <c r="G80" s="149"/>
+      <c r="F80" s="152"/>
+      <c r="G80" s="177"/>
     </row>
     <row r="81" spans="2:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B81" s="100" t="s">

</xml_diff>